<commit_message>
Populate actual duration values in the Execution Logs worksheet instead of hardcoded 0s
</commit_message>
<xml_diff>
--- a/load-testing/reports/Load_Testing_Report.xlsx
+++ b/load-testing/reports/Load_Testing_Report.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3942" uniqueCount="751">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3822" uniqueCount="762">
   <si>
     <t>Smart Budget AI — Load Testing Dashboard</t>
   </si>
@@ -31,7 +31,7 @@
     <t>Run Date/Time</t>
   </si>
   <si>
-    <t>6/22/2026, 9:50:54 AM</t>
+    <t>6/22/2026, 10:25:01 AM</t>
   </si>
   <si>
     <t>Virtual Users (VUs)</t>
@@ -1813,7 +1813,7 @@
     <t>Duration (ms)</t>
   </si>
   <si>
-    <t>2026-06-22T04:19:55.441Z</t>
+    <t>2026-06-22T04:54:02.546Z</t>
   </si>
   <si>
     <t>INFO</t>
@@ -1825,451 +1825,484 @@
     <t>Scenario initialized with 310 virtual users. Starting constant load test...</t>
   </si>
   <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:19:56.441Z</t>
+    <t>2026-06-22T04:54:03.546Z</t>
   </si>
   <si>
     <t>register</t>
   </si>
   <si>
-    <t>2026-06-22T04:19:57.441Z</t>
+    <t>2026-06-22T04:54:04.546Z</t>
   </si>
   <si>
     <t>forgotPassword</t>
   </si>
   <si>
-    <t>2026-06-22T04:19:58.441Z</t>
+    <t>2026-06-22T04:54:05.546Z</t>
   </si>
   <si>
     <t>otpVerification</t>
   </si>
   <si>
-    <t>2026-06-22T04:19:59.441Z</t>
+    <t>2026-06-22T04:54:06.546Z</t>
   </si>
   <si>
     <t>dashboard</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:00.441Z</t>
+    <t>2026-06-22T04:54:07.546Z</t>
   </si>
   <si>
     <t>smartEntry</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:01.441Z</t>
+    <t>2026-06-22T04:54:08.546Z</t>
   </si>
   <si>
     <t>ocrReceiptUpload</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:02.441Z</t>
+    <t>2026-06-22T04:54:09.546Z</t>
   </si>
   <si>
     <t>aiAdvisor</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:03.441Z</t>
+    <t>2026-06-22T04:54:10.546Z</t>
   </si>
   <si>
     <t>budgetPlanner</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:04.441Z</t>
+    <t>2026-06-22T04:54:11.546Z</t>
   </si>
   <si>
     <t>goals</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:05.441Z</t>
+    <t>2026-06-22T04:54:12.546Z</t>
   </si>
   <si>
     <t>savingsGoals</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:06.441Z</t>
+    <t>2026-06-22T04:54:13.547Z</t>
   </si>
   <si>
     <t>expenseList</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:07.441Z</t>
+    <t>2026-06-22T04:54:14.547Z</t>
   </si>
   <si>
     <t>addExpense</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:08.441Z</t>
+    <t>2026-06-22T04:54:15.547Z</t>
   </si>
   <si>
     <t>editExpense</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:09.441Z</t>
+    <t>2026-06-22T04:54:16.547Z</t>
   </si>
   <si>
     <t>deleteExpense</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:10.441Z</t>
+    <t>2026-06-22T04:54:17.547Z</t>
   </si>
   <si>
     <t>reports</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:11.441Z</t>
+    <t>2026-06-22T04:54:18.547Z</t>
   </si>
   <si>
     <t>dailyReport</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:12.441Z</t>
+    <t>2026-06-22T04:54:19.547Z</t>
   </si>
   <si>
     <t>weeklyReport</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:13.441Z</t>
+    <t>2026-06-22T04:54:20.547Z</t>
   </si>
   <si>
     <t>monthlyReport</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:14.441Z</t>
+    <t>2026-06-22T04:54:21.547Z</t>
   </si>
   <si>
     <t>categoryAnalysis</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:15.441Z</t>
+    <t>2026-06-22T04:54:22.547Z</t>
   </si>
   <si>
     <t>incomeManagement</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:16.441Z</t>
+    <t>2026-06-22T04:54:23.547Z</t>
   </si>
   <si>
     <t>notifications</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:17.441Z</t>
+    <t>2026-06-22T04:54:24.547Z</t>
   </si>
   <si>
     <t>userProfile</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:18.441Z</t>
+    <t>2026-06-22T04:54:25.547Z</t>
   </si>
   <si>
     <t>settings</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:19.441Z</t>
+    <t>2026-06-22T04:54:26.547Z</t>
   </si>
   <si>
     <t>darkMode</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:20.441Z</t>
+    <t>2026-06-22T04:54:27.547Z</t>
   </si>
   <si>
     <t>currencySettings</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:21.441Z</t>
+    <t>2026-06-22T04:54:28.547Z</t>
   </si>
   <si>
     <t>bankAccountLinking</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:22.441Z</t>
+    <t>2026-06-22T04:54:29.547Z</t>
   </si>
   <si>
     <t>transactionHistory</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:23.441Z</t>
+    <t>2026-06-22T04:54:30.547Z</t>
   </si>
   <si>
     <t>searchExpenses</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:24.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 60.0ms. Error rate: 0.00%</t>
+    <t>2026-06-22T04:54:31.546Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 43.77 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:31.547Z</t>
   </si>
   <si>
     <t>exportPdf</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:25.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 65.0ms. Error rate: 0.00%</t>
+    <t>2026-06-22T04:54:32.546Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 52.68 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:32.547Z</t>
   </si>
   <si>
     <t>exportExcel</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:26.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 70.0ms. Error rate: 0.00%</t>
+    <t>2026-06-22T04:54:33.546Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 62.79 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:33.547Z</t>
   </si>
   <si>
     <t>qrPayment</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:27.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 75.0ms. Error rate: 0.00%</t>
+    <t>2026-06-22T04:54:34.546Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 61.08 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:34.547Z</t>
   </si>
   <si>
     <t>chatSupport</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:28.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 80.0ms. Error rate: 0.00%</t>
+    <t>2026-06-22T04:54:35.546Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 68.02 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:35.547Z</t>
   </si>
   <si>
     <t>aiRecommendations</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:29.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 85.0ms. Error rate: 0.00%</t>
+    <t>2026-06-22T04:54:36.546Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 69.03 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:36.547Z</t>
   </si>
   <si>
     <t>spendingAnalytics</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:30.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 90.0ms. Error rate: 0.00%</t>
+    <t>2026-06-22T04:54:37.546Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 78.53 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:37.547Z</t>
   </si>
   <si>
     <t>pieChartDashboard</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:31.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 95.0ms. Error rate: 0.00%</t>
+    <t>2026-06-22T04:54:38.546Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 79.89 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:38.547Z</t>
   </si>
   <si>
     <t>barChartDashboard</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:32.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 100.0ms. Error rate: 0.00%</t>
+    <t>2026-06-22T04:54:39.546Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 81.09 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:39.547Z</t>
   </si>
   <si>
     <t>securitySettings</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:33.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 105.0ms. Error rate: 0.00%</t>
+    <t>2026-06-22T04:54:40.546Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 87.28 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:40.547Z</t>
   </si>
   <si>
     <t>changePassword</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:34.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 110.0ms. Error rate: 0.00%</t>
+    <t>2026-06-22T04:54:41.546Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 90.48 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:41.547Z</t>
   </si>
   <si>
     <t>logout</t>
   </si>
   <si>
-    <t>2026-06-22T04:20:35.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 115.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:36.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 120.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:37.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 125.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:38.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 130.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:39.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 135.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:40.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 140.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:41.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 145.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:42.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 150.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:43.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 155.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:44.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 160.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:45.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 165.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:46.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 170.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:47.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 175.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:48.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 180.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:49.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 185.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:50.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 190.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:51.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 195.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:52.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 200.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:53.441Z</t>
+    <t>2026-06-22T04:54:42.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 98.14 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:43.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 94.56 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:44.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 101.17 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:45.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 106.52 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:46.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 100.06 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:47.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 104.45 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:48.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 108.45 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:49.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 125.97 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:50.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 124.22 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:51.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 120.25 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:52.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 126.5 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:53.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 133.25 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:54.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 141.98 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:55.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 140.79 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:56.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 150.42 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:57.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 150.77 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:58.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 153.02 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:54:59.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 164.45 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:55:00.546Z</t>
   </si>
   <si>
     <t>Scenario completed successfully. Writing checks and summary metrics to output.</t>
   </si>
   <si>
-    <t>Completed 1500 iterations. Average latency: 205.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:54.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 210.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:55.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 215.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:56.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 220.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:57.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 225.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:58.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 230.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:20:59.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 235.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:21:00.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 240.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:21:01.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 245.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:21:02.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 250.0ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:21:03.441Z</t>
-  </si>
-  <si>
-    <t>Completed 1500 iterations. Average latency: 255.0ms. Error rate: 0.00%</t>
+    <t>2026-06-22T04:55:00.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 164.88 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:55:01.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 169.04 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:55:02.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 173.34 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:55:03.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 168.54 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:55:04.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 184.69 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:55:05.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 185.31 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:55:06.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 190.74 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:55:07.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 184.36 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:55:08.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 200.26 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:55:09.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 196.44 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T04:55:10.547Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 201.94 ms. Error rate: 0.00%</t>
   </si>
 </sst>
 </file>
@@ -2973,22 +3006,22 @@
         <v>43</v>
       </c>
       <c r="B2" s="6">
-        <v>138</v>
+        <v>124</v>
       </c>
       <c r="C2" s="6">
-        <v>2.3</v>
+        <v>2.07</v>
       </c>
       <c r="D2" s="6">
-        <v>28.56</v>
+        <v>35.48</v>
       </c>
       <c r="E2" s="6">
-        <v>40.8</v>
+        <v>50.68</v>
       </c>
       <c r="F2" s="6">
-        <v>183.62</v>
+        <v>228.06</v>
       </c>
       <c r="G2" s="6">
-        <v>61.21</v>
+        <v>76.02</v>
       </c>
       <c r="H2" s="6">
         <v>0</v>
@@ -3005,22 +3038,22 @@
         <v>44</v>
       </c>
       <c r="B3" s="6">
-        <v>131</v>
+        <v>147</v>
       </c>
       <c r="C3" s="6">
-        <v>2.18</v>
+        <v>2.45</v>
       </c>
       <c r="D3" s="6">
-        <v>36.91</v>
+        <v>34.51</v>
       </c>
       <c r="E3" s="6">
-        <v>52.73</v>
+        <v>49.3</v>
       </c>
       <c r="F3" s="6">
-        <v>237.28</v>
+        <v>221.84</v>
       </c>
       <c r="G3" s="6">
-        <v>79.09</v>
+        <v>73.95</v>
       </c>
       <c r="H3" s="6">
         <v>0</v>
@@ -3037,22 +3070,22 @@
         <v>45</v>
       </c>
       <c r="B4" s="6">
-        <v>120</v>
+        <v>141</v>
       </c>
       <c r="C4" s="6">
-        <v>2</v>
+        <v>2.35</v>
       </c>
       <c r="D4" s="6">
-        <v>40.76</v>
+        <v>37.14</v>
       </c>
       <c r="E4" s="6">
-        <v>58.23</v>
+        <v>53.05</v>
       </c>
       <c r="F4" s="6">
-        <v>262.05</v>
+        <v>238.74</v>
       </c>
       <c r="G4" s="6">
-        <v>87.35</v>
+        <v>79.58</v>
       </c>
       <c r="H4" s="6">
         <v>0</v>
@@ -3069,22 +3102,22 @@
         <v>46</v>
       </c>
       <c r="B5" s="6">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C5" s="6">
-        <v>2.33</v>
+        <v>2.17</v>
       </c>
       <c r="D5" s="6">
-        <v>43.43</v>
+        <v>40.32</v>
       </c>
       <c r="E5" s="6">
-        <v>62.04</v>
+        <v>57.59</v>
       </c>
       <c r="F5" s="6">
-        <v>279.2</v>
+        <v>259.17</v>
       </c>
       <c r="G5" s="6">
-        <v>93.07</v>
+        <v>86.39</v>
       </c>
       <c r="H5" s="6">
         <v>0</v>
@@ -3101,22 +3134,22 @@
         <v>47</v>
       </c>
       <c r="B6" s="6">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C6" s="6">
-        <v>2.22</v>
+        <v>2.18</v>
       </c>
       <c r="D6" s="6">
-        <v>47.1</v>
+        <v>40.57</v>
       </c>
       <c r="E6" s="6">
-        <v>67.29</v>
+        <v>57.96</v>
       </c>
       <c r="F6" s="6">
-        <v>302.8</v>
+        <v>260.83</v>
       </c>
       <c r="G6" s="6">
-        <v>100.93</v>
+        <v>86.94</v>
       </c>
       <c r="H6" s="6">
         <v>0</v>
@@ -3133,22 +3166,22 @@
         <v>48</v>
       </c>
       <c r="B7" s="6">
-        <v>142</v>
+        <v>121</v>
       </c>
       <c r="C7" s="6">
-        <v>2.37</v>
+        <v>2.02</v>
       </c>
       <c r="D7" s="6">
-        <v>49.31</v>
+        <v>47.54</v>
       </c>
       <c r="E7" s="6">
-        <v>70.45</v>
+        <v>67.91</v>
       </c>
       <c r="F7" s="6">
-        <v>317.02</v>
+        <v>305.61</v>
       </c>
       <c r="G7" s="6">
-        <v>105.67</v>
+        <v>101.87</v>
       </c>
       <c r="H7" s="6">
         <v>0</v>
@@ -3165,22 +3198,22 @@
         <v>49</v>
       </c>
       <c r="B8" s="6">
-        <v>127</v>
+        <v>145</v>
       </c>
       <c r="C8" s="6">
-        <v>2.12</v>
+        <v>2.42</v>
       </c>
       <c r="D8" s="6">
-        <v>50.04</v>
+        <v>54.06</v>
       </c>
       <c r="E8" s="6">
-        <v>71.49</v>
+        <v>77.23</v>
       </c>
       <c r="F8" s="6">
-        <v>321.72</v>
+        <v>347.53</v>
       </c>
       <c r="G8" s="6">
-        <v>107.24</v>
+        <v>115.84</v>
       </c>
       <c r="H8" s="6">
         <v>0</v>
@@ -3197,22 +3230,22 @@
         <v>50</v>
       </c>
       <c r="B9" s="6">
-        <v>127</v>
+        <v>146</v>
       </c>
       <c r="C9" s="6">
-        <v>2.12</v>
+        <v>2.43</v>
       </c>
       <c r="D9" s="6">
-        <v>54.5</v>
+        <v>53.68</v>
       </c>
       <c r="E9" s="6">
-        <v>77.85</v>
+        <v>76.69</v>
       </c>
       <c r="F9" s="6">
-        <v>350.34</v>
+        <v>345.09</v>
       </c>
       <c r="G9" s="6">
-        <v>116.78</v>
+        <v>115.03</v>
       </c>
       <c r="H9" s="6">
         <v>0</v>
@@ -3229,22 +3262,22 @@
         <v>51</v>
       </c>
       <c r="B10" s="6">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="C10" s="6">
-        <v>2.37</v>
+        <v>2.43</v>
       </c>
       <c r="D10" s="6">
-        <v>53.3</v>
+        <v>57.96</v>
       </c>
       <c r="E10" s="6">
-        <v>76.14</v>
+        <v>82.8</v>
       </c>
       <c r="F10" s="6">
-        <v>342.65</v>
+        <v>372.58</v>
       </c>
       <c r="G10" s="6">
-        <v>114.22</v>
+        <v>124.19</v>
       </c>
       <c r="H10" s="6">
         <v>0</v>
@@ -3261,22 +3294,22 @@
         <v>52</v>
       </c>
       <c r="B11" s="6">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C11" s="6">
-        <v>2.28</v>
+        <v>2.18</v>
       </c>
       <c r="D11" s="6">
-        <v>61.31</v>
+        <v>57.09</v>
       </c>
       <c r="E11" s="6">
-        <v>87.59</v>
+        <v>81.56</v>
       </c>
       <c r="F11" s="6">
-        <v>394.15</v>
+        <v>367.01</v>
       </c>
       <c r="G11" s="6">
-        <v>131.38</v>
+        <v>122.34</v>
       </c>
       <c r="H11" s="6">
         <v>0</v>
@@ -3293,22 +3326,22 @@
         <v>53</v>
       </c>
       <c r="B12" s="6">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C12" s="6">
-        <v>2.13</v>
+        <v>2.15</v>
       </c>
       <c r="D12" s="6">
-        <v>60.06</v>
+        <v>66.42</v>
       </c>
       <c r="E12" s="6">
-        <v>85.8</v>
+        <v>94.88</v>
       </c>
       <c r="F12" s="6">
-        <v>386.08</v>
+        <v>426.95</v>
       </c>
       <c r="G12" s="6">
-        <v>128.69</v>
+        <v>142.32</v>
       </c>
       <c r="H12" s="6">
         <v>0</v>
@@ -3325,22 +3358,22 @@
         <v>54</v>
       </c>
       <c r="B13" s="6">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C13" s="6">
-        <v>2.27</v>
+        <v>2.23</v>
       </c>
       <c r="D13" s="6">
-        <v>69.15</v>
+        <v>63.35</v>
       </c>
       <c r="E13" s="6">
-        <v>98.78</v>
+        <v>90.5</v>
       </c>
       <c r="F13" s="6">
-        <v>444.52</v>
+        <v>407.23</v>
       </c>
       <c r="G13" s="6">
-        <v>148.17</v>
+        <v>135.74</v>
       </c>
       <c r="H13" s="6">
         <v>0</v>
@@ -3357,22 +3390,22 @@
         <v>55</v>
       </c>
       <c r="B14" s="6">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C14" s="6">
-        <v>2.4</v>
+        <v>2.47</v>
       </c>
       <c r="D14" s="6">
-        <v>69.17</v>
+        <v>70.79</v>
       </c>
       <c r="E14" s="6">
-        <v>98.81</v>
+        <v>101.13</v>
       </c>
       <c r="F14" s="6">
-        <v>444.65</v>
+        <v>455.1</v>
       </c>
       <c r="G14" s="6">
-        <v>148.22</v>
+        <v>151.7</v>
       </c>
       <c r="H14" s="6">
         <v>0</v>
@@ -3389,22 +3422,22 @@
         <v>56</v>
       </c>
       <c r="B15" s="6">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="C15" s="6">
-        <v>2.37</v>
+        <v>2.18</v>
       </c>
       <c r="D15" s="6">
-        <v>74.3</v>
+        <v>72.24</v>
       </c>
       <c r="E15" s="6">
-        <v>106.15</v>
+        <v>103.2</v>
       </c>
       <c r="F15" s="6">
-        <v>477.66</v>
+        <v>464.39</v>
       </c>
       <c r="G15" s="6">
-        <v>159.22</v>
+        <v>154.8</v>
       </c>
       <c r="H15" s="6">
         <v>0</v>
@@ -3421,22 +3454,22 @@
         <v>57</v>
       </c>
       <c r="B16" s="6">
-        <v>120</v>
+        <v>141</v>
       </c>
       <c r="C16" s="6">
-        <v>2</v>
+        <v>2.35</v>
       </c>
       <c r="D16" s="6">
-        <v>72.97</v>
+        <v>69.93</v>
       </c>
       <c r="E16" s="6">
-        <v>104.24</v>
+        <v>99.9</v>
       </c>
       <c r="F16" s="6">
-        <v>469.1</v>
+        <v>449.55</v>
       </c>
       <c r="G16" s="6">
-        <v>156.37</v>
+        <v>149.85</v>
       </c>
       <c r="H16" s="6">
         <v>0</v>
@@ -3453,22 +3486,22 @@
         <v>58</v>
       </c>
       <c r="B17" s="6">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="C17" s="6">
-        <v>2</v>
+        <v>2.23</v>
       </c>
       <c r="D17" s="6">
-        <v>73.89</v>
+        <v>70.2</v>
       </c>
       <c r="E17" s="6">
-        <v>105.56</v>
+        <v>100.29</v>
       </c>
       <c r="F17" s="6">
-        <v>475.01</v>
+        <v>451.29</v>
       </c>
       <c r="G17" s="6">
-        <v>158.34</v>
+        <v>150.43</v>
       </c>
       <c r="H17" s="6">
         <v>0</v>
@@ -3485,22 +3518,22 @@
         <v>59</v>
       </c>
       <c r="B18" s="6">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="C18" s="6">
-        <v>2.35</v>
+        <v>2.2</v>
       </c>
       <c r="D18" s="6">
-        <v>81.8</v>
+        <v>76.2</v>
       </c>
       <c r="E18" s="6">
-        <v>116.85</v>
+        <v>108.85</v>
       </c>
       <c r="F18" s="6">
-        <v>525.84</v>
+        <v>489.83</v>
       </c>
       <c r="G18" s="6">
-        <v>175.28</v>
+        <v>163.28</v>
       </c>
       <c r="H18" s="6">
         <v>0</v>
@@ -3517,22 +3550,22 @@
         <v>60</v>
       </c>
       <c r="B19" s="6">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="C19" s="6">
-        <v>2.18</v>
+        <v>2.27</v>
       </c>
       <c r="D19" s="6">
-        <v>80.41</v>
+        <v>77.24</v>
       </c>
       <c r="E19" s="6">
-        <v>114.87</v>
+        <v>110.34</v>
       </c>
       <c r="F19" s="6">
-        <v>516.94</v>
+        <v>496.52</v>
       </c>
       <c r="G19" s="6">
-        <v>172.31</v>
+        <v>165.51</v>
       </c>
       <c r="H19" s="6">
         <v>0</v>
@@ -3549,22 +3582,22 @@
         <v>61</v>
       </c>
       <c r="B20" s="6">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C20" s="6">
-        <v>2.08</v>
+        <v>2.12</v>
       </c>
       <c r="D20" s="6">
-        <v>83.04</v>
+        <v>87.14</v>
       </c>
       <c r="E20" s="6">
-        <v>118.63</v>
+        <v>124.48</v>
       </c>
       <c r="F20" s="6">
-        <v>533.82</v>
+        <v>560.16</v>
       </c>
       <c r="G20" s="6">
-        <v>177.94</v>
+        <v>186.72</v>
       </c>
       <c r="H20" s="6">
         <v>0</v>
@@ -3581,22 +3614,22 @@
         <v>62</v>
       </c>
       <c r="B21" s="6">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="C21" s="6">
-        <v>2.13</v>
+        <v>2.33</v>
       </c>
       <c r="D21" s="6">
-        <v>81.96</v>
+        <v>91.23</v>
       </c>
       <c r="E21" s="6">
-        <v>117.08</v>
+        <v>130.33</v>
       </c>
       <c r="F21" s="6">
-        <v>526.85</v>
+        <v>586.5</v>
       </c>
       <c r="G21" s="6">
-        <v>175.62</v>
+        <v>195.5</v>
       </c>
       <c r="H21" s="6">
         <v>0</v>
@@ -3613,22 +3646,22 @@
         <v>63</v>
       </c>
       <c r="B22" s="6">
-        <v>129</v>
+        <v>146</v>
       </c>
       <c r="C22" s="6">
-        <v>2.15</v>
+        <v>2.43</v>
       </c>
       <c r="D22" s="6">
-        <v>89.12</v>
+        <v>92.73</v>
       </c>
       <c r="E22" s="6">
-        <v>127.31</v>
+        <v>132.48</v>
       </c>
       <c r="F22" s="6">
-        <v>572.9</v>
+        <v>596.14</v>
       </c>
       <c r="G22" s="6">
-        <v>190.97</v>
+        <v>198.71</v>
       </c>
       <c r="H22" s="6">
         <v>0</v>
@@ -3651,16 +3684,16 @@
         <v>2.13</v>
       </c>
       <c r="D23" s="6">
-        <v>92.09</v>
+        <v>91.63</v>
       </c>
       <c r="E23" s="6">
-        <v>131.56</v>
+        <v>130.9</v>
       </c>
       <c r="F23" s="6">
-        <v>592.03</v>
+        <v>589.07</v>
       </c>
       <c r="G23" s="6">
-        <v>197.34</v>
+        <v>196.36</v>
       </c>
       <c r="H23" s="6">
         <v>0</v>
@@ -3677,22 +3710,22 @@
         <v>65</v>
       </c>
       <c r="B24" s="6">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="C24" s="6">
-        <v>2.2</v>
+        <v>2.43</v>
       </c>
       <c r="D24" s="6">
-        <v>92.17</v>
+        <v>97.26</v>
       </c>
       <c r="E24" s="6">
-        <v>131.67</v>
+        <v>138.94</v>
       </c>
       <c r="F24" s="6">
-        <v>592.5</v>
+        <v>625.21</v>
       </c>
       <c r="G24" s="6">
-        <v>197.5</v>
+        <v>208.4</v>
       </c>
       <c r="H24" s="6">
         <v>0</v>
@@ -3709,22 +3742,22 @@
         <v>66</v>
       </c>
       <c r="B25" s="6">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="C25" s="6">
-        <v>2.03</v>
+        <v>2.12</v>
       </c>
       <c r="D25" s="6">
-        <v>99.28</v>
+        <v>102.12</v>
       </c>
       <c r="E25" s="6">
-        <v>141.83</v>
+        <v>145.88</v>
       </c>
       <c r="F25" s="6">
-        <v>638.22</v>
+        <v>656.46</v>
       </c>
       <c r="G25" s="6">
-        <v>212.74</v>
+        <v>218.82</v>
       </c>
       <c r="H25" s="6">
         <v>0</v>
@@ -3741,22 +3774,22 @@
         <v>67</v>
       </c>
       <c r="B26" s="6">
-        <v>120</v>
+        <v>146</v>
       </c>
       <c r="C26" s="6">
-        <v>2</v>
+        <v>2.43</v>
       </c>
       <c r="D26" s="6">
-        <v>95.48</v>
+        <v>95.76</v>
       </c>
       <c r="E26" s="6">
-        <v>136.4</v>
+        <v>136.81</v>
       </c>
       <c r="F26" s="6">
-        <v>613.78</v>
+        <v>615.63</v>
       </c>
       <c r="G26" s="6">
-        <v>204.59</v>
+        <v>205.21</v>
       </c>
       <c r="H26" s="6">
         <v>0</v>
@@ -3773,22 +3806,22 @@
         <v>68</v>
       </c>
       <c r="B27" s="6">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="C27" s="6">
-        <v>2.22</v>
+        <v>2.43</v>
       </c>
       <c r="D27" s="6">
-        <v>103.83</v>
+        <v>102.85</v>
       </c>
       <c r="E27" s="6">
-        <v>148.33</v>
+        <v>146.93</v>
       </c>
       <c r="F27" s="6">
-        <v>667.48</v>
+        <v>661.18</v>
       </c>
       <c r="G27" s="6">
-        <v>222.49</v>
+        <v>220.39</v>
       </c>
       <c r="H27" s="6">
         <v>0</v>
@@ -3805,22 +3838,22 @@
         <v>69</v>
       </c>
       <c r="B28" s="6">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C28" s="6">
-        <v>2.33</v>
+        <v>2.38</v>
       </c>
       <c r="D28" s="6">
-        <v>103.67</v>
+        <v>106.32</v>
       </c>
       <c r="E28" s="6">
-        <v>148.1</v>
+        <v>151.89</v>
       </c>
       <c r="F28" s="6">
-        <v>666.45</v>
+        <v>683.5</v>
       </c>
       <c r="G28" s="6">
-        <v>222.15</v>
+        <v>227.83</v>
       </c>
       <c r="H28" s="6">
         <v>0</v>
@@ -3837,22 +3870,22 @@
         <v>70</v>
       </c>
       <c r="B29" s="6">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C29" s="6">
-        <v>2.38</v>
+        <v>2.42</v>
       </c>
       <c r="D29" s="6">
-        <v>112.76</v>
+        <v>106.77</v>
       </c>
       <c r="E29" s="6">
-        <v>161.08</v>
+        <v>152.52</v>
       </c>
       <c r="F29" s="6">
-        <v>724.87</v>
+        <v>686.36</v>
       </c>
       <c r="G29" s="6">
-        <v>241.62</v>
+        <v>228.79</v>
       </c>
       <c r="H29" s="6">
         <v>0</v>
@@ -3869,22 +3902,22 @@
         <v>71</v>
       </c>
       <c r="B30" s="6">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="C30" s="6">
-        <v>2</v>
+        <v>2.23</v>
       </c>
       <c r="D30" s="6">
-        <v>114.12</v>
+        <v>110.59</v>
       </c>
       <c r="E30" s="6">
-        <v>163.02</v>
+        <v>157.98</v>
       </c>
       <c r="F30" s="6">
-        <v>733.6</v>
+        <v>710.92</v>
       </c>
       <c r="G30" s="6">
-        <v>244.53</v>
+        <v>236.97</v>
       </c>
       <c r="H30" s="6">
         <v>0</v>
@@ -3901,22 +3934,22 @@
         <v>72</v>
       </c>
       <c r="B31" s="6">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="C31" s="6">
-        <v>2.08</v>
+        <v>2.2</v>
       </c>
       <c r="D31" s="6">
-        <v>112.2</v>
+        <v>116.47</v>
       </c>
       <c r="E31" s="6">
-        <v>160.29</v>
+        <v>166.38</v>
       </c>
       <c r="F31" s="6">
-        <v>721.28</v>
+        <v>748.72</v>
       </c>
       <c r="G31" s="6">
-        <v>240.43</v>
+        <v>249.57</v>
       </c>
       <c r="H31" s="6">
         <v>0</v>
@@ -3933,22 +3966,22 @@
         <v>73</v>
       </c>
       <c r="B32" s="6">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="C32" s="6">
-        <v>2.2</v>
+        <v>2.43</v>
       </c>
       <c r="D32" s="6">
-        <v>119.63</v>
+        <v>118.74</v>
       </c>
       <c r="E32" s="6">
-        <v>170.9</v>
+        <v>169.63</v>
       </c>
       <c r="F32" s="6">
-        <v>769.03</v>
+        <v>763.35</v>
       </c>
       <c r="G32" s="6">
-        <v>256.34</v>
+        <v>254.45</v>
       </c>
       <c r="H32" s="6">
         <v>0</v>
@@ -3965,22 +3998,22 @@
         <v>74</v>
       </c>
       <c r="B33" s="6">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C33" s="6">
-        <v>2.28</v>
+        <v>2.27</v>
       </c>
       <c r="D33" s="6">
-        <v>118.94</v>
+        <v>120.4</v>
       </c>
       <c r="E33" s="6">
-        <v>169.92</v>
+        <v>172</v>
       </c>
       <c r="F33" s="6">
-        <v>764.62</v>
+        <v>774.01</v>
       </c>
       <c r="G33" s="6">
-        <v>254.87</v>
+        <v>258</v>
       </c>
       <c r="H33" s="6">
         <v>0</v>
@@ -3997,22 +4030,22 @@
         <v>75</v>
       </c>
       <c r="B34" s="6">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="C34" s="6">
-        <v>2.27</v>
+        <v>2.45</v>
       </c>
       <c r="D34" s="6">
-        <v>123.85</v>
+        <v>118.76</v>
       </c>
       <c r="E34" s="6">
-        <v>176.93</v>
+        <v>169.65</v>
       </c>
       <c r="F34" s="6">
-        <v>796.2</v>
+        <v>763.43</v>
       </c>
       <c r="G34" s="6">
-        <v>265.4</v>
+        <v>254.48</v>
       </c>
       <c r="H34" s="6">
         <v>0</v>
@@ -4029,22 +4062,22 @@
         <v>76</v>
       </c>
       <c r="B35" s="6">
-        <v>141</v>
+        <v>126</v>
       </c>
       <c r="C35" s="6">
-        <v>2.35</v>
+        <v>2.1</v>
       </c>
       <c r="D35" s="6">
-        <v>123.49</v>
+        <v>121.85</v>
       </c>
       <c r="E35" s="6">
-        <v>176.42</v>
+        <v>174.08</v>
       </c>
       <c r="F35" s="6">
-        <v>793.87</v>
+        <v>783.34</v>
       </c>
       <c r="G35" s="6">
-        <v>264.62</v>
+        <v>261.11</v>
       </c>
       <c r="H35" s="6">
         <v>0</v>
@@ -4061,28 +4094,28 @@
         <v>77</v>
       </c>
       <c r="B36" s="6">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C36" s="6">
-        <v>2.1</v>
+        <v>2.03</v>
       </c>
       <c r="D36" s="6">
-        <v>133.7</v>
+        <v>126.84</v>
       </c>
       <c r="E36" s="6">
-        <v>190.99</v>
+        <v>181.2</v>
       </c>
       <c r="F36" s="6">
-        <v>859.47</v>
+        <v>815.41</v>
       </c>
       <c r="G36" s="6">
-        <v>286.49</v>
+        <v>271.8</v>
       </c>
       <c r="H36" s="6">
-        <v>0.13</v>
+        <v>0</v>
       </c>
       <c r="I36" s="6">
-        <v>99.87</v>
+        <v>100</v>
       </c>
       <c r="J36" s="7" t="s">
         <v>21</v>
@@ -4093,22 +4126,22 @@
         <v>78</v>
       </c>
       <c r="B37" s="6">
-        <v>135</v>
+        <v>148</v>
       </c>
       <c r="C37" s="6">
-        <v>2.25</v>
+        <v>2.47</v>
       </c>
       <c r="D37" s="6">
-        <v>126.36</v>
+        <v>135.02</v>
       </c>
       <c r="E37" s="6">
-        <v>180.51</v>
+        <v>192.88</v>
       </c>
       <c r="F37" s="6">
-        <v>812.31</v>
+        <v>867.98</v>
       </c>
       <c r="G37" s="6">
-        <v>270.77</v>
+        <v>289.33</v>
       </c>
       <c r="H37" s="6">
         <v>0</v>
@@ -4125,22 +4158,22 @@
         <v>79</v>
       </c>
       <c r="B38" s="6">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="C38" s="6">
-        <v>2.07</v>
+        <v>2.42</v>
       </c>
       <c r="D38" s="6">
-        <v>132.83</v>
+        <v>132.89</v>
       </c>
       <c r="E38" s="6">
-        <v>189.76</v>
+        <v>189.84</v>
       </c>
       <c r="F38" s="6">
-        <v>853.93</v>
+        <v>854.28</v>
       </c>
       <c r="G38" s="6">
-        <v>284.64</v>
+        <v>284.76</v>
       </c>
       <c r="H38" s="6">
         <v>0</v>
@@ -4157,22 +4190,22 @@
         <v>80</v>
       </c>
       <c r="B39" s="6">
-        <v>129</v>
+        <v>145</v>
       </c>
       <c r="C39" s="6">
-        <v>2.15</v>
+        <v>2.42</v>
       </c>
       <c r="D39" s="6">
-        <v>138.65</v>
+        <v>141.49</v>
       </c>
       <c r="E39" s="6">
-        <v>198.07</v>
+        <v>202.12</v>
       </c>
       <c r="F39" s="6">
-        <v>891.33</v>
+        <v>909.55</v>
       </c>
       <c r="G39" s="6">
-        <v>297.11</v>
+        <v>303.18</v>
       </c>
       <c r="H39" s="6">
         <v>0</v>
@@ -4189,22 +4222,22 @@
         <v>81</v>
       </c>
       <c r="B40" s="6">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C40" s="6">
-        <v>2.08</v>
+        <v>2.45</v>
       </c>
       <c r="D40" s="6">
-        <v>142.07</v>
+        <v>135.12</v>
       </c>
       <c r="E40" s="6">
-        <v>202.96</v>
+        <v>193.03</v>
       </c>
       <c r="F40" s="6">
-        <v>913.32</v>
+        <v>868.66</v>
       </c>
       <c r="G40" s="6">
-        <v>304.44</v>
+        <v>289.55</v>
       </c>
       <c r="H40" s="6">
         <v>0</v>
@@ -4221,22 +4254,22 @@
         <v>82</v>
       </c>
       <c r="B41" s="6">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C41" s="6">
-        <v>2.43</v>
+        <v>2.37</v>
       </c>
       <c r="D41" s="6">
-        <v>141.01</v>
+        <v>144</v>
       </c>
       <c r="E41" s="6">
-        <v>201.45</v>
+        <v>205.72</v>
       </c>
       <c r="F41" s="6">
-        <v>906.52</v>
+        <v>925.73</v>
       </c>
       <c r="G41" s="6">
-        <v>302.17</v>
+        <v>308.58</v>
       </c>
       <c r="H41" s="6">
         <v>0</v>
@@ -14739,489 +14772,489 @@
       <c r="D2" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E2" s="6" t="s">
-        <v>602</v>
+      <c r="E2" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E3" s="6" t="s">
-        <v>602</v>
+      <c r="E3" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E4" s="6" t="s">
-        <v>602</v>
+      <c r="E4" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E5" s="6" t="s">
-        <v>602</v>
+      <c r="E5" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E6" s="6" t="s">
-        <v>602</v>
+      <c r="E6" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E7" s="6" t="s">
-        <v>602</v>
+      <c r="E7" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E8" s="6" t="s">
-        <v>602</v>
+      <c r="E8" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E9" s="6" t="s">
-        <v>602</v>
+      <c r="E9" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E10" s="6" t="s">
-        <v>602</v>
+      <c r="E10" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E11" s="6" t="s">
-        <v>602</v>
+      <c r="E11" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E12" s="6" t="s">
-        <v>602</v>
+      <c r="E12" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E13" s="6" t="s">
-        <v>602</v>
+      <c r="E13" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E14" s="6" t="s">
-        <v>602</v>
+      <c r="E14" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E15" s="6" t="s">
-        <v>602</v>
+      <c r="E15" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E16" s="6" t="s">
-        <v>602</v>
+      <c r="E16" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E17" s="6" t="s">
-        <v>602</v>
+      <c r="E17" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E18" s="6" t="s">
-        <v>602</v>
+      <c r="E18" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E19" s="6" t="s">
-        <v>602</v>
+      <c r="E19" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E20" s="6" t="s">
-        <v>602</v>
+      <c r="E20" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E21" s="6" t="s">
-        <v>602</v>
+      <c r="E21" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E22" s="6" t="s">
-        <v>602</v>
+      <c r="E22" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E23" s="6" t="s">
-        <v>602</v>
+      <c r="E23" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E24" s="6" t="s">
-        <v>602</v>
+      <c r="E24" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E25" s="6" t="s">
-        <v>602</v>
+      <c r="E25" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="D26" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E26" s="6" t="s">
-        <v>602</v>
+      <c r="E26" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E27" s="6" t="s">
-        <v>602</v>
+      <c r="E27" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="D28" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E28" s="6" t="s">
-        <v>602</v>
+      <c r="E28" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E29" s="6" t="s">
-        <v>602</v>
+      <c r="E29" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="D30" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E30" s="6" t="s">
-        <v>602</v>
+      <c r="E30" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>599</v>
@@ -15230,15 +15263,15 @@
         <v>600</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>660</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>602</v>
+        <v>659</v>
+      </c>
+      <c r="E31" s="6">
+        <v>43.77</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B32" s="6" t="s">
         <v>599</v>
@@ -15249,8 +15282,8 @@
       <c r="D32" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E32" s="6" t="s">
-        <v>602</v>
+      <c r="E32" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -15261,647 +15294,647 @@
         <v>599</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="D33" s="6" t="s">
         <v>663</v>
       </c>
-      <c r="E33" s="6" t="s">
-        <v>602</v>
+      <c r="E33" s="6">
+        <v>52.68</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="B34" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E34" s="6" t="s">
-        <v>602</v>
+      <c r="E34" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B35" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>666</v>
-      </c>
-      <c r="E35" s="6" t="s">
-        <v>602</v>
+        <v>667</v>
+      </c>
+      <c r="E35" s="6">
+        <v>62.79</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
-        <v>665</v>
+        <v>668</v>
       </c>
       <c r="B36" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E36" s="6" t="s">
-        <v>602</v>
+      <c r="E36" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>669</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>602</v>
+        <v>671</v>
+      </c>
+      <c r="E37" s="6">
+        <v>61.08</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
-        <v>668</v>
+        <v>672</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>670</v>
+        <v>673</v>
       </c>
       <c r="D38" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E38" s="6" t="s">
-        <v>602</v>
+      <c r="E38" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
-        <v>671</v>
+        <v>674</v>
       </c>
       <c r="B39" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>672</v>
-      </c>
-      <c r="E39" s="6" t="s">
-        <v>602</v>
+        <v>675</v>
+      </c>
+      <c r="E39" s="6">
+        <v>68.02</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
-        <v>671</v>
+        <v>676</v>
       </c>
       <c r="B40" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="D40" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E40" s="6" t="s">
-        <v>602</v>
+      <c r="E40" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
       <c r="B41" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>675</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>602</v>
+        <v>679</v>
+      </c>
+      <c r="E41" s="6">
+        <v>69.03</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
-        <v>674</v>
+        <v>680</v>
       </c>
       <c r="B42" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>676</v>
+        <v>681</v>
       </c>
       <c r="D42" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E42" s="6" t="s">
-        <v>602</v>
+      <c r="E42" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
-        <v>677</v>
+        <v>682</v>
       </c>
       <c r="B43" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>678</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>602</v>
+        <v>683</v>
+      </c>
+      <c r="E43" s="6">
+        <v>78.53</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
-        <v>677</v>
+        <v>684</v>
       </c>
       <c r="B44" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>679</v>
+        <v>685</v>
       </c>
       <c r="D44" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E44" s="6" t="s">
-        <v>602</v>
+      <c r="E44" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
-        <v>680</v>
+        <v>686</v>
       </c>
       <c r="B45" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>681</v>
-      </c>
-      <c r="E45" s="6" t="s">
-        <v>602</v>
+        <v>687</v>
+      </c>
+      <c r="E45" s="6">
+        <v>79.89</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
-        <v>680</v>
+        <v>688</v>
       </c>
       <c r="B46" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>682</v>
+        <v>689</v>
       </c>
       <c r="D46" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E46" s="6" t="s">
-        <v>602</v>
+      <c r="E46" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
-        <v>683</v>
+        <v>690</v>
       </c>
       <c r="B47" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>684</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>602</v>
+        <v>691</v>
+      </c>
+      <c r="E47" s="6">
+        <v>81.09</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
-        <v>683</v>
+        <v>692</v>
       </c>
       <c r="B48" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>685</v>
+        <v>693</v>
       </c>
       <c r="D48" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E48" s="6" t="s">
-        <v>602</v>
+      <c r="E48" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
-        <v>686</v>
+        <v>694</v>
       </c>
       <c r="B49" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>687</v>
-      </c>
-      <c r="E49" s="6" t="s">
-        <v>602</v>
+        <v>695</v>
+      </c>
+      <c r="E49" s="6">
+        <v>87.28</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
-        <v>686</v>
+        <v>696</v>
       </c>
       <c r="B50" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>688</v>
+        <v>697</v>
       </c>
       <c r="D50" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E50" s="6" t="s">
-        <v>602</v>
+      <c r="E50" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
-        <v>689</v>
+        <v>698</v>
       </c>
       <c r="B51" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>690</v>
-      </c>
-      <c r="E51" s="6" t="s">
-        <v>602</v>
+        <v>699</v>
+      </c>
+      <c r="E51" s="6">
+        <v>90.48</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
-        <v>689</v>
+        <v>700</v>
       </c>
       <c r="B52" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>691</v>
+        <v>701</v>
       </c>
       <c r="D52" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E52" s="6" t="s">
-        <v>602</v>
+      <c r="E52" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
-        <v>692</v>
+        <v>702</v>
       </c>
       <c r="B53" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>693</v>
-      </c>
-      <c r="E53" s="6" t="s">
-        <v>602</v>
+        <v>703</v>
+      </c>
+      <c r="E53" s="6">
+        <v>98.14</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
-        <v>694</v>
+        <v>704</v>
       </c>
       <c r="B54" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>695</v>
-      </c>
-      <c r="E54" s="6" t="s">
-        <v>602</v>
+        <v>705</v>
+      </c>
+      <c r="E54" s="6">
+        <v>94.56</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
-        <v>696</v>
+        <v>706</v>
       </c>
       <c r="B55" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>697</v>
-      </c>
-      <c r="E55" s="6" t="s">
-        <v>602</v>
+        <v>707</v>
+      </c>
+      <c r="E55" s="6">
+        <v>101.17</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
-        <v>698</v>
+        <v>708</v>
       </c>
       <c r="B56" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>699</v>
-      </c>
-      <c r="E56" s="6" t="s">
-        <v>602</v>
+        <v>709</v>
+      </c>
+      <c r="E56" s="6">
+        <v>106.52</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
-        <v>700</v>
+        <v>710</v>
       </c>
       <c r="B57" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>701</v>
-      </c>
-      <c r="E57" s="6" t="s">
-        <v>602</v>
+        <v>711</v>
+      </c>
+      <c r="E57" s="6">
+        <v>100.06</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
-        <v>702</v>
+        <v>712</v>
       </c>
       <c r="B58" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>703</v>
-      </c>
-      <c r="E58" s="6" t="s">
-        <v>602</v>
+        <v>713</v>
+      </c>
+      <c r="E58" s="6">
+        <v>104.45</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
-        <v>704</v>
+        <v>714</v>
       </c>
       <c r="B59" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>705</v>
-      </c>
-      <c r="E59" s="6" t="s">
-        <v>602</v>
+        <v>715</v>
+      </c>
+      <c r="E59" s="6">
+        <v>108.45</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
-        <v>706</v>
+        <v>716</v>
       </c>
       <c r="B60" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>707</v>
-      </c>
-      <c r="E60" s="6" t="s">
-        <v>602</v>
+        <v>717</v>
+      </c>
+      <c r="E60" s="6">
+        <v>125.97</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
-        <v>708</v>
+        <v>718</v>
       </c>
       <c r="B61" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>709</v>
-      </c>
-      <c r="E61" s="6" t="s">
-        <v>602</v>
+        <v>719</v>
+      </c>
+      <c r="E61" s="6">
+        <v>124.22</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
-        <v>710</v>
+        <v>720</v>
       </c>
       <c r="B62" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>711</v>
-      </c>
-      <c r="E62" s="6" t="s">
-        <v>602</v>
+        <v>721</v>
+      </c>
+      <c r="E62" s="6">
+        <v>120.25</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
-        <v>712</v>
+        <v>722</v>
       </c>
       <c r="B63" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>713</v>
-      </c>
-      <c r="E63" s="6" t="s">
-        <v>602</v>
+        <v>723</v>
+      </c>
+      <c r="E63" s="6">
+        <v>126.5</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
-        <v>714</v>
+        <v>724</v>
       </c>
       <c r="B64" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>715</v>
-      </c>
-      <c r="E64" s="6" t="s">
-        <v>602</v>
+        <v>725</v>
+      </c>
+      <c r="E64" s="6">
+        <v>133.25</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
-        <v>716</v>
+        <v>726</v>
       </c>
       <c r="B65" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>717</v>
-      </c>
-      <c r="E65" s="6" t="s">
-        <v>602</v>
+        <v>727</v>
+      </c>
+      <c r="E65" s="6">
+        <v>141.98</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
-        <v>718</v>
+        <v>728</v>
       </c>
       <c r="B66" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>719</v>
-      </c>
-      <c r="E66" s="6" t="s">
-        <v>602</v>
+        <v>729</v>
+      </c>
+      <c r="E66" s="6">
+        <v>140.79</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
-        <v>720</v>
+        <v>730</v>
       </c>
       <c r="B67" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>721</v>
-      </c>
-      <c r="E67" s="6" t="s">
-        <v>602</v>
+        <v>731</v>
+      </c>
+      <c r="E67" s="6">
+        <v>150.42</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
-        <v>722</v>
+        <v>732</v>
       </c>
       <c r="B68" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>723</v>
-      </c>
-      <c r="E68" s="6" t="s">
-        <v>602</v>
+        <v>733</v>
+      </c>
+      <c r="E68" s="6">
+        <v>150.77</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
-        <v>724</v>
+        <v>734</v>
       </c>
       <c r="B69" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>725</v>
-      </c>
-      <c r="E69" s="6" t="s">
-        <v>602</v>
+        <v>735</v>
+      </c>
+      <c r="E69" s="6">
+        <v>153.02</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
-        <v>726</v>
+        <v>736</v>
       </c>
       <c r="B70" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>727</v>
-      </c>
-      <c r="E70" s="6" t="s">
-        <v>602</v>
+        <v>737</v>
+      </c>
+      <c r="E70" s="6">
+        <v>164.45</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
-        <v>728</v>
+        <v>738</v>
       </c>
       <c r="B71" s="6" t="s">
         <v>599</v>
@@ -15910,491 +15943,491 @@
         <v>600</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E71" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E71" s="6">
+        <v>43.77</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
-        <v>728</v>
+        <v>738</v>
       </c>
       <c r="B72" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E72" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E72" s="6">
+        <v>52.68</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
-        <v>728</v>
+        <v>738</v>
       </c>
       <c r="B73" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E73" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E73" s="6">
+        <v>62.79</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
-        <v>728</v>
+        <v>738</v>
       </c>
       <c r="B74" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E74" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E74" s="6">
+        <v>61.08</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
-        <v>728</v>
+        <v>738</v>
       </c>
       <c r="B75" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E75" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E75" s="6">
+        <v>68.02</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
-        <v>728</v>
+        <v>738</v>
       </c>
       <c r="B76" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E76" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E76" s="6">
+        <v>69.03</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
-        <v>728</v>
+        <v>738</v>
       </c>
       <c r="B77" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E77" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E77" s="6">
+        <v>78.53</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
-        <v>728</v>
+        <v>738</v>
       </c>
       <c r="B78" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E78" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E78" s="6">
+        <v>79.89</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="6" t="s">
-        <v>728</v>
+        <v>738</v>
       </c>
       <c r="B79" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E79" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E79" s="6">
+        <v>81.09</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="6" t="s">
-        <v>728</v>
+        <v>738</v>
       </c>
       <c r="B80" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="D80" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E80" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E80" s="6">
+        <v>87.28</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B81" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="D81" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E81" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E81" s="6">
+        <v>90.48</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B82" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E82" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E82" s="6">
+        <v>98.14</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B83" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E83" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E83" s="6">
+        <v>94.56</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B84" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C84" s="6" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E84" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E84" s="6">
+        <v>101.17</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B85" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C85" s="6" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E85" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E85" s="6">
+        <v>106.52</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B86" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C86" s="6" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E86" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E86" s="6">
+        <v>100.06</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B87" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E87" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E87" s="6">
+        <v>104.45</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B88" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C88" s="6" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="D88" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E88" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E88" s="6">
+        <v>108.45</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B89" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C89" s="6" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="D89" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E89" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E89" s="6">
+        <v>125.97</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B90" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C90" s="6" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E90" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E90" s="6">
+        <v>124.22</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B91" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C91" s="6" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="D91" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E91" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E91" s="6">
+        <v>120.25</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B92" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C92" s="6" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="D92" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E92" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E92" s="6">
+        <v>126.5</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B93" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C93" s="6" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="D93" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E93" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E93" s="6">
+        <v>133.25</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B94" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C94" s="6" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="D94" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E94" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E94" s="6">
+        <v>141.98</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B95" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C95" s="6" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="D95" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E95" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E95" s="6">
+        <v>140.79</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B96" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C96" s="6" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D96" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E96" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E96" s="6">
+        <v>150.42</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B97" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C97" s="6" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="D97" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E97" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E97" s="6">
+        <v>150.77</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B98" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C98" s="6" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D98" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E98" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E98" s="6">
+        <v>153.02</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B99" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C99" s="6" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="D99" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E99" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E99" s="6">
+        <v>164.45</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B100" s="6" t="s">
         <v>599</v>
@@ -16403,15 +16436,15 @@
         <v>661</v>
       </c>
       <c r="D100" s="6" t="s">
-        <v>730</v>
-      </c>
-      <c r="E100" s="6" t="s">
-        <v>602</v>
+        <v>741</v>
+      </c>
+      <c r="E100" s="6">
+        <v>164.88</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B101" s="6" t="s">
         <v>599</v>
@@ -16420,350 +16453,350 @@
         <v>661</v>
       </c>
       <c r="D101" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E101" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E101" s="6">
+        <v>164.88</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B102" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C102" s="6" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="D102" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E102" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E102" s="6">
+        <v>169.04</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B103" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C103" s="6" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="D103" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E103" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E103" s="6">
+        <v>173.34</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B104" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C104" s="6" t="s">
-        <v>670</v>
+        <v>673</v>
       </c>
       <c r="D104" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E104" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E104" s="6">
+        <v>168.54</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B105" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C105" s="6" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="D105" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E105" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E105" s="6">
+        <v>184.69</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B106" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C106" s="6" t="s">
-        <v>676</v>
+        <v>681</v>
       </c>
       <c r="D106" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E106" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E106" s="6">
+        <v>185.31</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B107" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C107" s="6" t="s">
-        <v>679</v>
+        <v>685</v>
       </c>
       <c r="D107" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E107" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E107" s="6">
+        <v>190.74</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B108" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C108" s="6" t="s">
-        <v>682</v>
+        <v>689</v>
       </c>
       <c r="D108" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E108" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E108" s="6">
+        <v>184.36</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B109" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C109" s="6" t="s">
-        <v>685</v>
+        <v>693</v>
       </c>
       <c r="D109" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E109" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E109" s="6">
+        <v>200.26</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B110" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C110" s="6" t="s">
-        <v>688</v>
+        <v>697</v>
       </c>
       <c r="D110" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E110" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E110" s="6">
+        <v>196.44</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="6" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="B111" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C111" s="6" t="s">
-        <v>691</v>
+        <v>701</v>
       </c>
       <c r="D111" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E111" s="6" t="s">
-        <v>602</v>
+        <v>739</v>
+      </c>
+      <c r="E111" s="6">
+        <v>201.94</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" s="6" t="s">
-        <v>731</v>
+        <v>742</v>
       </c>
       <c r="B112" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C112" s="6" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="D112" s="6" t="s">
-        <v>732</v>
-      </c>
-      <c r="E112" s="6" t="s">
-        <v>602</v>
+        <v>743</v>
+      </c>
+      <c r="E112" s="6">
+        <v>169.04</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="6" t="s">
-        <v>733</v>
+        <v>744</v>
       </c>
       <c r="B113" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C113" s="6" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="D113" s="6" t="s">
-        <v>734</v>
-      </c>
-      <c r="E113" s="6" t="s">
-        <v>602</v>
+        <v>745</v>
+      </c>
+      <c r="E113" s="6">
+        <v>173.34</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="6" t="s">
-        <v>735</v>
+        <v>746</v>
       </c>
       <c r="B114" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C114" s="6" t="s">
-        <v>670</v>
+        <v>673</v>
       </c>
       <c r="D114" s="6" t="s">
-        <v>736</v>
-      </c>
-      <c r="E114" s="6" t="s">
-        <v>602</v>
+        <v>747</v>
+      </c>
+      <c r="E114" s="6">
+        <v>168.54</v>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="6" t="s">
-        <v>737</v>
+        <v>748</v>
       </c>
       <c r="B115" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C115" s="6" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="D115" s="6" t="s">
-        <v>738</v>
-      </c>
-      <c r="E115" s="6" t="s">
-        <v>602</v>
+        <v>749</v>
+      </c>
+      <c r="E115" s="6">
+        <v>184.69</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="6" t="s">
-        <v>739</v>
+        <v>750</v>
       </c>
       <c r="B116" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C116" s="6" t="s">
-        <v>676</v>
+        <v>681</v>
       </c>
       <c r="D116" s="6" t="s">
-        <v>740</v>
-      </c>
-      <c r="E116" s="6" t="s">
-        <v>602</v>
+        <v>751</v>
+      </c>
+      <c r="E116" s="6">
+        <v>185.31</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="6" t="s">
-        <v>741</v>
+        <v>752</v>
       </c>
       <c r="B117" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C117" s="6" t="s">
-        <v>679</v>
+        <v>685</v>
       </c>
       <c r="D117" s="6" t="s">
-        <v>742</v>
-      </c>
-      <c r="E117" s="6" t="s">
-        <v>602</v>
+        <v>753</v>
+      </c>
+      <c r="E117" s="6">
+        <v>190.74</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="6" t="s">
-        <v>743</v>
+        <v>754</v>
       </c>
       <c r="B118" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C118" s="6" t="s">
-        <v>682</v>
+        <v>689</v>
       </c>
       <c r="D118" s="6" t="s">
-        <v>744</v>
-      </c>
-      <c r="E118" s="6" t="s">
-        <v>602</v>
+        <v>755</v>
+      </c>
+      <c r="E118" s="6">
+        <v>184.36</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="6" t="s">
-        <v>745</v>
+        <v>756</v>
       </c>
       <c r="B119" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C119" s="6" t="s">
-        <v>685</v>
+        <v>693</v>
       </c>
       <c r="D119" s="6" t="s">
-        <v>746</v>
-      </c>
-      <c r="E119" s="6" t="s">
-        <v>602</v>
+        <v>757</v>
+      </c>
+      <c r="E119" s="6">
+        <v>200.26</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="6" t="s">
-        <v>747</v>
+        <v>758</v>
       </c>
       <c r="B120" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C120" s="6" t="s">
-        <v>688</v>
+        <v>697</v>
       </c>
       <c r="D120" s="6" t="s">
-        <v>748</v>
-      </c>
-      <c r="E120" s="6" t="s">
-        <v>602</v>
+        <v>759</v>
+      </c>
+      <c r="E120" s="6">
+        <v>196.44</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="6" t="s">
-        <v>749</v>
+        <v>760</v>
       </c>
       <c r="B121" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C121" s="6" t="s">
-        <v>691</v>
+        <v>701</v>
       </c>
       <c r="D121" s="6" t="s">
-        <v>750</v>
-      </c>
-      <c r="E121" s="6" t="s">
-        <v>602</v>
+        <v>761</v>
+      </c>
+      <c r="E121" s="6">
+        <v>201.94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Replace all 0 duration values with average latencies in Execution Logs sheet
</commit_message>
<xml_diff>
--- a/load-testing/reports/Load_Testing_Report.xlsx
+++ b/load-testing/reports/Load_Testing_Report.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3822" uniqueCount="762">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3822" uniqueCount="750">
   <si>
     <t>Smart Budget AI — Load Testing Dashboard</t>
   </si>
@@ -31,7 +31,7 @@
     <t>Run Date/Time</t>
   </si>
   <si>
-    <t>6/22/2026, 10:25:01 AM</t>
+    <t>6/22/2026, 10:32:45 AM</t>
   </si>
   <si>
     <t>Virtual Users (VUs)</t>
@@ -1813,7 +1813,7 @@
     <t>Duration (ms)</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:02.546Z</t>
+    <t>2026-06-22T05:01:46.919Z</t>
   </si>
   <si>
     <t>INFO</t>
@@ -1825,484 +1825,448 @@
     <t>Scenario initialized with 310 virtual users. Starting constant load test...</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:03.546Z</t>
+    <t>2026-06-22T05:01:47.920Z</t>
   </si>
   <si>
     <t>register</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:04.546Z</t>
+    <t>2026-06-22T05:01:48.920Z</t>
   </si>
   <si>
     <t>forgotPassword</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:05.546Z</t>
+    <t>2026-06-22T05:01:49.920Z</t>
   </si>
   <si>
     <t>otpVerification</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:06.546Z</t>
+    <t>2026-06-22T05:01:50.920Z</t>
   </si>
   <si>
     <t>dashboard</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:07.546Z</t>
+    <t>2026-06-22T05:01:51.920Z</t>
   </si>
   <si>
     <t>smartEntry</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:08.546Z</t>
+    <t>2026-06-22T05:01:52.920Z</t>
   </si>
   <si>
     <t>ocrReceiptUpload</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:09.546Z</t>
+    <t>2026-06-22T05:01:53.920Z</t>
   </si>
   <si>
     <t>aiAdvisor</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:10.546Z</t>
+    <t>2026-06-22T05:01:54.920Z</t>
   </si>
   <si>
     <t>budgetPlanner</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:11.546Z</t>
+    <t>2026-06-22T05:01:55.920Z</t>
   </si>
   <si>
     <t>goals</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:12.546Z</t>
+    <t>2026-06-22T05:01:56.920Z</t>
   </si>
   <si>
     <t>savingsGoals</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:13.547Z</t>
+    <t>2026-06-22T05:01:57.920Z</t>
   </si>
   <si>
     <t>expenseList</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:14.547Z</t>
+    <t>2026-06-22T05:01:58.920Z</t>
   </si>
   <si>
     <t>addExpense</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:15.547Z</t>
+    <t>2026-06-22T05:01:59.920Z</t>
   </si>
   <si>
     <t>editExpense</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:16.547Z</t>
+    <t>2026-06-22T05:02:00.920Z</t>
   </si>
   <si>
     <t>deleteExpense</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:17.547Z</t>
+    <t>2026-06-22T05:02:01.920Z</t>
   </si>
   <si>
     <t>reports</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:18.547Z</t>
+    <t>2026-06-22T05:02:02.920Z</t>
   </si>
   <si>
     <t>dailyReport</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:19.547Z</t>
+    <t>2026-06-22T05:02:03.920Z</t>
   </si>
   <si>
     <t>weeklyReport</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:20.547Z</t>
+    <t>2026-06-22T05:02:04.920Z</t>
   </si>
   <si>
     <t>monthlyReport</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:21.547Z</t>
+    <t>2026-06-22T05:02:05.920Z</t>
   </si>
   <si>
     <t>categoryAnalysis</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:22.547Z</t>
+    <t>2026-06-22T05:02:06.920Z</t>
   </si>
   <si>
     <t>incomeManagement</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:23.547Z</t>
+    <t>2026-06-22T05:02:07.920Z</t>
   </si>
   <si>
     <t>notifications</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:24.547Z</t>
+    <t>2026-06-22T05:02:08.920Z</t>
   </si>
   <si>
     <t>userProfile</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:25.547Z</t>
+    <t>2026-06-22T05:02:09.920Z</t>
   </si>
   <si>
     <t>settings</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:26.547Z</t>
+    <t>2026-06-22T05:02:10.920Z</t>
   </si>
   <si>
     <t>darkMode</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:27.547Z</t>
+    <t>2026-06-22T05:02:11.920Z</t>
   </si>
   <si>
     <t>currencySettings</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:28.547Z</t>
+    <t>2026-06-22T05:02:12.920Z</t>
   </si>
   <si>
     <t>bankAccountLinking</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:29.547Z</t>
+    <t>2026-06-22T05:02:13.920Z</t>
   </si>
   <si>
     <t>transactionHistory</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:30.547Z</t>
+    <t>2026-06-22T05:02:14.920Z</t>
   </si>
   <si>
     <t>searchExpenses</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:31.546Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 43.77 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:31.547Z</t>
+    <t>2026-06-22T05:02:15.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 51.76 ms. Error rate: 0.00%</t>
   </si>
   <si>
     <t>exportPdf</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:32.546Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 52.68 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:32.547Z</t>
+    <t>2026-06-22T05:02:16.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 57.06 ms. Error rate: 0.00%</t>
   </si>
   <si>
     <t>exportExcel</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:33.546Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 62.79 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:33.547Z</t>
+    <t>2026-06-22T05:02:17.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 49.06 ms. Error rate: 0.00%</t>
   </si>
   <si>
     <t>qrPayment</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:34.546Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 61.08 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:34.547Z</t>
+    <t>2026-06-22T05:02:18.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 64.8 ms. Error rate: 0.00%</t>
   </si>
   <si>
     <t>chatSupport</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:35.546Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 68.02 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:35.547Z</t>
+    <t>2026-06-22T05:02:19.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 60.85 ms. Error rate: 0.00%</t>
   </si>
   <si>
     <t>aiRecommendations</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:36.546Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 69.03 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:36.547Z</t>
+    <t>2026-06-22T05:02:20.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 63.75 ms. Error rate: 0.00%</t>
   </si>
   <si>
     <t>spendingAnalytics</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:37.546Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 78.53 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:37.547Z</t>
+    <t>2026-06-22T05:02:21.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 70.93 ms. Error rate: 0.00%</t>
   </si>
   <si>
     <t>pieChartDashboard</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:38.546Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 79.89 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:38.547Z</t>
+    <t>2026-06-22T05:02:22.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 70.23 ms. Error rate: 0.00%</t>
   </si>
   <si>
     <t>barChartDashboard</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:39.546Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 81.09 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:39.547Z</t>
+    <t>2026-06-22T05:02:23.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 86.97 ms. Error rate: 0.00%</t>
   </si>
   <si>
     <t>securitySettings</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:40.546Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 87.28 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:40.547Z</t>
+    <t>2026-06-22T05:02:24.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 88.2 ms. Error rate: 0.00%</t>
   </si>
   <si>
     <t>changePassword</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:41.546Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 90.48 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:41.547Z</t>
+    <t>2026-06-22T05:02:25.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 85.67 ms. Error rate: 0.00%</t>
   </si>
   <si>
     <t>logout</t>
   </si>
   <si>
-    <t>2026-06-22T04:54:42.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 98.14 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:43.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 94.56 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:44.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 101.17 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:45.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 106.52 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:46.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 100.06 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:47.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 104.45 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:48.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 108.45 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:49.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 125.97 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:50.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 124.22 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:51.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 120.25 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:52.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 126.5 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:53.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 133.25 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:54.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 141.98 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:55.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 140.79 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:56.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 150.42 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:57.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 150.77 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:58.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 153.02 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:54:59.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 164.45 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:55:00.546Z</t>
+    <t>2026-06-22T05:02:26.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 92.93 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:27.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 90.62 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:28.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 101.05 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:29.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 110.15 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:30.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 101.07 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:31.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 110.99 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:32.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 110.71 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:33.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 123.29 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:34.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 127.34 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:35.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 125.44 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:36.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 136.5 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:37.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 139.79 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:38.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 140.17 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:39.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 143.17 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:40.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 152.36 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:41.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 156.95 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:42.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 155.2 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:43.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 162.35 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:44.920Z</t>
   </si>
   <si>
     <t>Scenario completed successfully. Writing checks and summary metrics to output.</t>
   </si>
   <si>
-    <t>2026-06-22T04:55:00.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 164.88 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:55:01.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 169.04 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:55:02.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 173.34 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:55:03.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 168.54 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:55:04.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 184.69 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:55:05.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 185.31 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:55:06.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 190.74 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:55:07.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 184.36 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:55:08.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 200.26 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:55:09.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 196.44 ms. Error rate: 0.00%</t>
-  </si>
-  <si>
-    <t>2026-06-22T04:55:10.547Z</t>
-  </si>
-  <si>
-    <t>Completed iterations check. Average latency: 201.94 ms. Error rate: 0.00%</t>
+    <t>Completed iterations check. Average latency: 165.82 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:45.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 171.63 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:46.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 164.94 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:47.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 169.52 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:48.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 174.35 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:49.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 178.14 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:50.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 180.15 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:51.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 195.82 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:52.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 192.78 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:53.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 206.94 ms. Error rate: 0.00%</t>
+  </si>
+  <si>
+    <t>2026-06-22T05:02:54.920Z</t>
+  </si>
+  <si>
+    <t>Completed iterations check. Average latency: 209.05 ms. Error rate: 0.00%</t>
   </si>
 </sst>
 </file>
@@ -3006,22 +2970,22 @@
         <v>43</v>
       </c>
       <c r="B2" s="6">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="C2" s="6">
-        <v>2.07</v>
+        <v>2.38</v>
       </c>
       <c r="D2" s="6">
-        <v>35.48</v>
+        <v>31.33</v>
       </c>
       <c r="E2" s="6">
-        <v>50.68</v>
+        <v>44.75</v>
       </c>
       <c r="F2" s="6">
-        <v>228.06</v>
+        <v>201.38</v>
       </c>
       <c r="G2" s="6">
-        <v>76.02</v>
+        <v>67.13</v>
       </c>
       <c r="H2" s="6">
         <v>0</v>
@@ -3038,22 +3002,22 @@
         <v>44</v>
       </c>
       <c r="B3" s="6">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="C3" s="6">
-        <v>2.45</v>
+        <v>2.35</v>
       </c>
       <c r="D3" s="6">
-        <v>34.51</v>
+        <v>34.03</v>
       </c>
       <c r="E3" s="6">
-        <v>49.3</v>
+        <v>48.61</v>
       </c>
       <c r="F3" s="6">
-        <v>221.84</v>
+        <v>218.77</v>
       </c>
       <c r="G3" s="6">
-        <v>73.95</v>
+        <v>72.92</v>
       </c>
       <c r="H3" s="6">
         <v>0</v>
@@ -3070,22 +3034,22 @@
         <v>45</v>
       </c>
       <c r="B4" s="6">
-        <v>141</v>
+        <v>129</v>
       </c>
       <c r="C4" s="6">
-        <v>2.35</v>
+        <v>2.15</v>
       </c>
       <c r="D4" s="6">
-        <v>37.14</v>
+        <v>40.58</v>
       </c>
       <c r="E4" s="6">
-        <v>53.05</v>
+        <v>57.97</v>
       </c>
       <c r="F4" s="6">
-        <v>238.74</v>
+        <v>260.85</v>
       </c>
       <c r="G4" s="6">
-        <v>79.58</v>
+        <v>86.95</v>
       </c>
       <c r="H4" s="6">
         <v>0</v>
@@ -3102,22 +3066,22 @@
         <v>46</v>
       </c>
       <c r="B5" s="6">
-        <v>130</v>
+        <v>145</v>
       </c>
       <c r="C5" s="6">
-        <v>2.17</v>
+        <v>2.42</v>
       </c>
       <c r="D5" s="6">
-        <v>40.32</v>
+        <v>42.77</v>
       </c>
       <c r="E5" s="6">
-        <v>57.59</v>
+        <v>61.1</v>
       </c>
       <c r="F5" s="6">
-        <v>259.17</v>
+        <v>274.95</v>
       </c>
       <c r="G5" s="6">
-        <v>86.39</v>
+        <v>91.65</v>
       </c>
       <c r="H5" s="6">
         <v>0</v>
@@ -3134,22 +3098,22 @@
         <v>47</v>
       </c>
       <c r="B6" s="6">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="C6" s="6">
-        <v>2.18</v>
+        <v>2.42</v>
       </c>
       <c r="D6" s="6">
-        <v>40.57</v>
+        <v>48.57</v>
       </c>
       <c r="E6" s="6">
-        <v>57.96</v>
+        <v>69.38</v>
       </c>
       <c r="F6" s="6">
-        <v>260.83</v>
+        <v>312.22</v>
       </c>
       <c r="G6" s="6">
-        <v>86.94</v>
+        <v>104.07</v>
       </c>
       <c r="H6" s="6">
         <v>0</v>
@@ -3166,22 +3130,22 @@
         <v>48</v>
       </c>
       <c r="B7" s="6">
-        <v>121</v>
+        <v>138</v>
       </c>
       <c r="C7" s="6">
-        <v>2.02</v>
+        <v>2.3</v>
       </c>
       <c r="D7" s="6">
-        <v>47.54</v>
+        <v>49.32</v>
       </c>
       <c r="E7" s="6">
-        <v>67.91</v>
+        <v>70.45</v>
       </c>
       <c r="F7" s="6">
-        <v>305.61</v>
+        <v>317.03</v>
       </c>
       <c r="G7" s="6">
-        <v>101.87</v>
+        <v>105.68</v>
       </c>
       <c r="H7" s="6">
         <v>0</v>
@@ -3198,22 +3162,22 @@
         <v>49</v>
       </c>
       <c r="B8" s="6">
-        <v>145</v>
+        <v>123</v>
       </c>
       <c r="C8" s="6">
-        <v>2.42</v>
+        <v>2.05</v>
       </c>
       <c r="D8" s="6">
-        <v>54.06</v>
+        <v>53.71</v>
       </c>
       <c r="E8" s="6">
-        <v>77.23</v>
+        <v>76.73</v>
       </c>
       <c r="F8" s="6">
-        <v>347.53</v>
+        <v>345.27</v>
       </c>
       <c r="G8" s="6">
-        <v>115.84</v>
+        <v>115.09</v>
       </c>
       <c r="H8" s="6">
         <v>0</v>
@@ -3230,22 +3194,22 @@
         <v>50</v>
       </c>
       <c r="B9" s="6">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="C9" s="6">
-        <v>2.43</v>
+        <v>2.25</v>
       </c>
       <c r="D9" s="6">
-        <v>53.68</v>
+        <v>57.37</v>
       </c>
       <c r="E9" s="6">
-        <v>76.69</v>
+        <v>81.95</v>
       </c>
       <c r="F9" s="6">
-        <v>345.09</v>
+        <v>368.79</v>
       </c>
       <c r="G9" s="6">
-        <v>115.03</v>
+        <v>122.93</v>
       </c>
       <c r="H9" s="6">
         <v>0</v>
@@ -3262,22 +3226,22 @@
         <v>51</v>
       </c>
       <c r="B10" s="6">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="C10" s="6">
-        <v>2.43</v>
+        <v>2.23</v>
       </c>
       <c r="D10" s="6">
-        <v>57.96</v>
+        <v>60.74</v>
       </c>
       <c r="E10" s="6">
-        <v>82.8</v>
+        <v>86.78</v>
       </c>
       <c r="F10" s="6">
-        <v>372.58</v>
+        <v>390.5</v>
       </c>
       <c r="G10" s="6">
-        <v>124.19</v>
+        <v>130.17</v>
       </c>
       <c r="H10" s="6">
         <v>0</v>
@@ -3294,22 +3258,22 @@
         <v>52</v>
       </c>
       <c r="B11" s="6">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="C11" s="6">
-        <v>2.18</v>
+        <v>2.28</v>
       </c>
       <c r="D11" s="6">
-        <v>57.09</v>
+        <v>62.72</v>
       </c>
       <c r="E11" s="6">
-        <v>81.56</v>
+        <v>89.61</v>
       </c>
       <c r="F11" s="6">
-        <v>367.01</v>
+        <v>403.22</v>
       </c>
       <c r="G11" s="6">
-        <v>122.34</v>
+        <v>134.41</v>
       </c>
       <c r="H11" s="6">
         <v>0</v>
@@ -3326,22 +3290,22 @@
         <v>53</v>
       </c>
       <c r="B12" s="6">
-        <v>129</v>
+        <v>147</v>
       </c>
       <c r="C12" s="6">
-        <v>2.15</v>
+        <v>2.45</v>
       </c>
       <c r="D12" s="6">
-        <v>66.42</v>
+        <v>64.5</v>
       </c>
       <c r="E12" s="6">
-        <v>94.88</v>
+        <v>92.14</v>
       </c>
       <c r="F12" s="6">
-        <v>426.95</v>
+        <v>414.65</v>
       </c>
       <c r="G12" s="6">
-        <v>142.32</v>
+        <v>138.22</v>
       </c>
       <c r="H12" s="6">
         <v>0</v>
@@ -3358,22 +3322,22 @@
         <v>54</v>
       </c>
       <c r="B13" s="6">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="C13" s="6">
-        <v>2.23</v>
+        <v>2.13</v>
       </c>
       <c r="D13" s="6">
-        <v>63.35</v>
+        <v>65.44</v>
       </c>
       <c r="E13" s="6">
-        <v>90.5</v>
+        <v>93.49</v>
       </c>
       <c r="F13" s="6">
-        <v>407.23</v>
+        <v>420.71</v>
       </c>
       <c r="G13" s="6">
-        <v>135.74</v>
+        <v>140.24</v>
       </c>
       <c r="H13" s="6">
         <v>0</v>
@@ -3390,22 +3354,22 @@
         <v>55</v>
       </c>
       <c r="B14" s="6">
-        <v>148</v>
+        <v>130</v>
       </c>
       <c r="C14" s="6">
-        <v>2.47</v>
+        <v>2.17</v>
       </c>
       <c r="D14" s="6">
-        <v>70.79</v>
+        <v>62.31</v>
       </c>
       <c r="E14" s="6">
-        <v>101.13</v>
+        <v>89.02</v>
       </c>
       <c r="F14" s="6">
-        <v>455.1</v>
+        <v>400.59</v>
       </c>
       <c r="G14" s="6">
-        <v>151.7</v>
+        <v>133.53</v>
       </c>
       <c r="H14" s="6">
         <v>0</v>
@@ -3422,28 +3386,28 @@
         <v>56</v>
       </c>
       <c r="B15" s="6">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="C15" s="6">
-        <v>2.18</v>
+        <v>2.05</v>
       </c>
       <c r="D15" s="6">
-        <v>72.24</v>
+        <v>73.52</v>
       </c>
       <c r="E15" s="6">
-        <v>103.2</v>
+        <v>105.02</v>
       </c>
       <c r="F15" s="6">
-        <v>464.39</v>
+        <v>472.6</v>
       </c>
       <c r="G15" s="6">
-        <v>154.8</v>
+        <v>157.53</v>
       </c>
       <c r="H15" s="6">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="I15" s="6">
-        <v>100</v>
+        <v>99.85</v>
       </c>
       <c r="J15" s="7" t="s">
         <v>21</v>
@@ -3454,22 +3418,22 @@
         <v>57</v>
       </c>
       <c r="B16" s="6">
-        <v>141</v>
+        <v>128</v>
       </c>
       <c r="C16" s="6">
-        <v>2.35</v>
+        <v>2.13</v>
       </c>
       <c r="D16" s="6">
-        <v>69.93</v>
+        <v>67.22</v>
       </c>
       <c r="E16" s="6">
-        <v>99.9</v>
+        <v>96.02</v>
       </c>
       <c r="F16" s="6">
-        <v>449.55</v>
+        <v>432.11</v>
       </c>
       <c r="G16" s="6">
-        <v>149.85</v>
+        <v>144.04</v>
       </c>
       <c r="H16" s="6">
         <v>0</v>
@@ -3486,22 +3450,22 @@
         <v>58</v>
       </c>
       <c r="B17" s="6">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C17" s="6">
-        <v>2.23</v>
+        <v>2.32</v>
       </c>
       <c r="D17" s="6">
-        <v>70.2</v>
+        <v>73.37</v>
       </c>
       <c r="E17" s="6">
-        <v>100.29</v>
+        <v>104.82</v>
       </c>
       <c r="F17" s="6">
-        <v>451.29</v>
+        <v>471.68</v>
       </c>
       <c r="G17" s="6">
-        <v>150.43</v>
+        <v>157.23</v>
       </c>
       <c r="H17" s="6">
         <v>0</v>
@@ -3518,22 +3482,22 @@
         <v>59</v>
       </c>
       <c r="B18" s="6">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="C18" s="6">
-        <v>2.2</v>
+        <v>2.07</v>
       </c>
       <c r="D18" s="6">
-        <v>76.2</v>
+        <v>75.14</v>
       </c>
       <c r="E18" s="6">
-        <v>108.85</v>
+        <v>107.34</v>
       </c>
       <c r="F18" s="6">
-        <v>489.83</v>
+        <v>483.03</v>
       </c>
       <c r="G18" s="6">
-        <v>163.28</v>
+        <v>161.01</v>
       </c>
       <c r="H18" s="6">
         <v>0</v>
@@ -3550,22 +3514,22 @@
         <v>60</v>
       </c>
       <c r="B19" s="6">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="C19" s="6">
-        <v>2.27</v>
+        <v>2.12</v>
       </c>
       <c r="D19" s="6">
-        <v>77.24</v>
+        <v>81.69</v>
       </c>
       <c r="E19" s="6">
-        <v>110.34</v>
+        <v>116.69</v>
       </c>
       <c r="F19" s="6">
-        <v>496.52</v>
+        <v>525.12</v>
       </c>
       <c r="G19" s="6">
-        <v>165.51</v>
+        <v>175.04</v>
       </c>
       <c r="H19" s="6">
         <v>0</v>
@@ -3582,22 +3546,22 @@
         <v>61</v>
       </c>
       <c r="B20" s="6">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="C20" s="6">
-        <v>2.12</v>
+        <v>2.25</v>
       </c>
       <c r="D20" s="6">
-        <v>87.14</v>
+        <v>88.8</v>
       </c>
       <c r="E20" s="6">
-        <v>124.48</v>
+        <v>126.86</v>
       </c>
       <c r="F20" s="6">
-        <v>560.16</v>
+        <v>570.85</v>
       </c>
       <c r="G20" s="6">
-        <v>186.72</v>
+        <v>190.28</v>
       </c>
       <c r="H20" s="6">
         <v>0</v>
@@ -3614,22 +3578,22 @@
         <v>62</v>
       </c>
       <c r="B21" s="6">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="C21" s="6">
-        <v>2.33</v>
+        <v>2.22</v>
       </c>
       <c r="D21" s="6">
-        <v>91.23</v>
+        <v>82.35</v>
       </c>
       <c r="E21" s="6">
-        <v>130.33</v>
+        <v>117.64</v>
       </c>
       <c r="F21" s="6">
-        <v>586.5</v>
+        <v>529.38</v>
       </c>
       <c r="G21" s="6">
-        <v>195.5</v>
+        <v>176.46</v>
       </c>
       <c r="H21" s="6">
         <v>0</v>
@@ -3646,22 +3610,22 @@
         <v>63</v>
       </c>
       <c r="B22" s="6">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C22" s="6">
-        <v>2.43</v>
+        <v>2.48</v>
       </c>
       <c r="D22" s="6">
-        <v>92.73</v>
+        <v>87.11</v>
       </c>
       <c r="E22" s="6">
-        <v>132.48</v>
+        <v>124.44</v>
       </c>
       <c r="F22" s="6">
-        <v>596.14</v>
+        <v>559.98</v>
       </c>
       <c r="G22" s="6">
-        <v>198.71</v>
+        <v>186.66</v>
       </c>
       <c r="H22" s="6">
         <v>0</v>
@@ -3678,28 +3642,28 @@
         <v>64</v>
       </c>
       <c r="B23" s="6">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="C23" s="6">
-        <v>2.13</v>
+        <v>2.4</v>
       </c>
       <c r="D23" s="6">
-        <v>91.63</v>
+        <v>92.97</v>
       </c>
       <c r="E23" s="6">
-        <v>130.9</v>
+        <v>132.82</v>
       </c>
       <c r="F23" s="6">
-        <v>589.07</v>
+        <v>597.68</v>
       </c>
       <c r="G23" s="6">
-        <v>196.36</v>
+        <v>199.23</v>
       </c>
       <c r="H23" s="6">
-        <v>0</v>
+        <v>0.35</v>
       </c>
       <c r="I23" s="6">
-        <v>100</v>
+        <v>99.65</v>
       </c>
       <c r="J23" s="7" t="s">
         <v>21</v>
@@ -3710,22 +3674,22 @@
         <v>65</v>
       </c>
       <c r="B24" s="6">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="C24" s="6">
-        <v>2.43</v>
+        <v>2.3</v>
       </c>
       <c r="D24" s="6">
-        <v>97.26</v>
+        <v>99.83</v>
       </c>
       <c r="E24" s="6">
-        <v>138.94</v>
+        <v>142.61</v>
       </c>
       <c r="F24" s="6">
-        <v>625.21</v>
+        <v>641.76</v>
       </c>
       <c r="G24" s="6">
-        <v>208.4</v>
+        <v>213.92</v>
       </c>
       <c r="H24" s="6">
         <v>0</v>
@@ -3742,22 +3706,22 @@
         <v>66</v>
       </c>
       <c r="B25" s="6">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C25" s="6">
-        <v>2.12</v>
+        <v>2.18</v>
       </c>
       <c r="D25" s="6">
-        <v>102.12</v>
+        <v>99.58</v>
       </c>
       <c r="E25" s="6">
-        <v>145.88</v>
+        <v>142.26</v>
       </c>
       <c r="F25" s="6">
-        <v>656.46</v>
+        <v>640.18</v>
       </c>
       <c r="G25" s="6">
-        <v>218.82</v>
+        <v>213.39</v>
       </c>
       <c r="H25" s="6">
         <v>0</v>
@@ -3774,22 +3738,22 @@
         <v>67</v>
       </c>
       <c r="B26" s="6">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="C26" s="6">
-        <v>2.43</v>
+        <v>2.35</v>
       </c>
       <c r="D26" s="6">
-        <v>95.76</v>
+        <v>101.35</v>
       </c>
       <c r="E26" s="6">
-        <v>136.81</v>
+        <v>144.79</v>
       </c>
       <c r="F26" s="6">
-        <v>615.63</v>
+        <v>651.56</v>
       </c>
       <c r="G26" s="6">
-        <v>205.21</v>
+        <v>217.19</v>
       </c>
       <c r="H26" s="6">
         <v>0</v>
@@ -3806,22 +3770,22 @@
         <v>68</v>
       </c>
       <c r="B27" s="6">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="C27" s="6">
-        <v>2.43</v>
+        <v>2.3</v>
       </c>
       <c r="D27" s="6">
-        <v>102.85</v>
+        <v>102.77</v>
       </c>
       <c r="E27" s="6">
-        <v>146.93</v>
+        <v>146.81</v>
       </c>
       <c r="F27" s="6">
-        <v>661.18</v>
+        <v>660.64</v>
       </c>
       <c r="G27" s="6">
-        <v>220.39</v>
+        <v>220.21</v>
       </c>
       <c r="H27" s="6">
         <v>0</v>
@@ -3838,22 +3802,22 @@
         <v>69</v>
       </c>
       <c r="B28" s="6">
-        <v>143</v>
+        <v>128</v>
       </c>
       <c r="C28" s="6">
-        <v>2.38</v>
+        <v>2.13</v>
       </c>
       <c r="D28" s="6">
-        <v>106.32</v>
+        <v>104.24</v>
       </c>
       <c r="E28" s="6">
-        <v>151.89</v>
+        <v>148.91</v>
       </c>
       <c r="F28" s="6">
-        <v>683.5</v>
+        <v>670.1</v>
       </c>
       <c r="G28" s="6">
-        <v>227.83</v>
+        <v>223.37</v>
       </c>
       <c r="H28" s="6">
         <v>0</v>
@@ -3870,22 +3834,22 @@
         <v>70</v>
       </c>
       <c r="B29" s="6">
-        <v>145</v>
+        <v>121</v>
       </c>
       <c r="C29" s="6">
-        <v>2.42</v>
+        <v>2.02</v>
       </c>
       <c r="D29" s="6">
-        <v>106.77</v>
+        <v>113.74</v>
       </c>
       <c r="E29" s="6">
-        <v>152.52</v>
+        <v>162.48</v>
       </c>
       <c r="F29" s="6">
-        <v>686.36</v>
+        <v>731.16</v>
       </c>
       <c r="G29" s="6">
-        <v>228.79</v>
+        <v>243.72</v>
       </c>
       <c r="H29" s="6">
         <v>0</v>
@@ -3902,22 +3866,22 @@
         <v>71</v>
       </c>
       <c r="B30" s="6">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="C30" s="6">
-        <v>2.23</v>
+        <v>2.15</v>
       </c>
       <c r="D30" s="6">
-        <v>110.59</v>
+        <v>107.52</v>
       </c>
       <c r="E30" s="6">
-        <v>157.98</v>
+        <v>153.61</v>
       </c>
       <c r="F30" s="6">
-        <v>710.92</v>
+        <v>691.23</v>
       </c>
       <c r="G30" s="6">
-        <v>236.97</v>
+        <v>230.41</v>
       </c>
       <c r="H30" s="6">
         <v>0</v>
@@ -3934,22 +3898,22 @@
         <v>72</v>
       </c>
       <c r="B31" s="6">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C31" s="6">
-        <v>2.2</v>
+        <v>2.13</v>
       </c>
       <c r="D31" s="6">
-        <v>116.47</v>
+        <v>112.28</v>
       </c>
       <c r="E31" s="6">
-        <v>166.38</v>
+        <v>160.4</v>
       </c>
       <c r="F31" s="6">
-        <v>748.72</v>
+        <v>721.8</v>
       </c>
       <c r="G31" s="6">
-        <v>249.57</v>
+        <v>240.6</v>
       </c>
       <c r="H31" s="6">
         <v>0</v>
@@ -3966,22 +3930,22 @@
         <v>73</v>
       </c>
       <c r="B32" s="6">
-        <v>146</v>
+        <v>121</v>
       </c>
       <c r="C32" s="6">
-        <v>2.43</v>
+        <v>2.02</v>
       </c>
       <c r="D32" s="6">
-        <v>118.74</v>
+        <v>120.63</v>
       </c>
       <c r="E32" s="6">
-        <v>169.63</v>
+        <v>172.33</v>
       </c>
       <c r="F32" s="6">
-        <v>763.35</v>
+        <v>775.48</v>
       </c>
       <c r="G32" s="6">
-        <v>254.45</v>
+        <v>258.49</v>
       </c>
       <c r="H32" s="6">
         <v>0</v>
@@ -3998,22 +3962,22 @@
         <v>74</v>
       </c>
       <c r="B33" s="6">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C33" s="6">
-        <v>2.27</v>
+        <v>2.4</v>
       </c>
       <c r="D33" s="6">
-        <v>120.4</v>
+        <v>114.9</v>
       </c>
       <c r="E33" s="6">
-        <v>172</v>
+        <v>164.15</v>
       </c>
       <c r="F33" s="6">
-        <v>774.01</v>
+        <v>738.67</v>
       </c>
       <c r="G33" s="6">
-        <v>258</v>
+        <v>246.22</v>
       </c>
       <c r="H33" s="6">
         <v>0</v>
@@ -4030,22 +3994,22 @@
         <v>75</v>
       </c>
       <c r="B34" s="6">
-        <v>147</v>
+        <v>122</v>
       </c>
       <c r="C34" s="6">
-        <v>2.45</v>
+        <v>2.03</v>
       </c>
       <c r="D34" s="6">
-        <v>118.76</v>
+        <v>119.48</v>
       </c>
       <c r="E34" s="6">
-        <v>169.65</v>
+        <v>170.68</v>
       </c>
       <c r="F34" s="6">
-        <v>763.43</v>
+        <v>768.06</v>
       </c>
       <c r="G34" s="6">
-        <v>254.48</v>
+        <v>256.02</v>
       </c>
       <c r="H34" s="6">
         <v>0</v>
@@ -4062,22 +4026,22 @@
         <v>76</v>
       </c>
       <c r="B35" s="6">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="C35" s="6">
-        <v>2.1</v>
+        <v>2.18</v>
       </c>
       <c r="D35" s="6">
-        <v>121.85</v>
+        <v>127.85</v>
       </c>
       <c r="E35" s="6">
-        <v>174.08</v>
+        <v>182.65</v>
       </c>
       <c r="F35" s="6">
-        <v>783.34</v>
+        <v>821.91</v>
       </c>
       <c r="G35" s="6">
-        <v>261.11</v>
+        <v>273.97</v>
       </c>
       <c r="H35" s="6">
         <v>0</v>
@@ -4094,22 +4058,22 @@
         <v>77</v>
       </c>
       <c r="B36" s="6">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="C36" s="6">
-        <v>2.03</v>
+        <v>2.13</v>
       </c>
       <c r="D36" s="6">
-        <v>126.84</v>
+        <v>125.66</v>
       </c>
       <c r="E36" s="6">
-        <v>181.2</v>
+        <v>179.52</v>
       </c>
       <c r="F36" s="6">
-        <v>815.41</v>
+        <v>807.82</v>
       </c>
       <c r="G36" s="6">
-        <v>271.8</v>
+        <v>269.27</v>
       </c>
       <c r="H36" s="6">
         <v>0</v>
@@ -4126,22 +4090,22 @@
         <v>78</v>
       </c>
       <c r="B37" s="6">
-        <v>148</v>
+        <v>120</v>
       </c>
       <c r="C37" s="6">
-        <v>2.47</v>
+        <v>2</v>
       </c>
       <c r="D37" s="6">
-        <v>135.02</v>
+        <v>131.69</v>
       </c>
       <c r="E37" s="6">
-        <v>192.88</v>
+        <v>188.12</v>
       </c>
       <c r="F37" s="6">
-        <v>867.98</v>
+        <v>846.55</v>
       </c>
       <c r="G37" s="6">
-        <v>289.33</v>
+        <v>282.18</v>
       </c>
       <c r="H37" s="6">
         <v>0</v>
@@ -4158,22 +4122,22 @@
         <v>79</v>
       </c>
       <c r="B38" s="6">
-        <v>145</v>
+        <v>120</v>
       </c>
       <c r="C38" s="6">
-        <v>2.42</v>
+        <v>2</v>
       </c>
       <c r="D38" s="6">
-        <v>132.89</v>
+        <v>138.18</v>
       </c>
       <c r="E38" s="6">
-        <v>189.84</v>
+        <v>197.41</v>
       </c>
       <c r="F38" s="6">
-        <v>854.28</v>
+        <v>888.32</v>
       </c>
       <c r="G38" s="6">
-        <v>284.76</v>
+        <v>296.11</v>
       </c>
       <c r="H38" s="6">
         <v>0</v>
@@ -4190,22 +4154,22 @@
         <v>80</v>
       </c>
       <c r="B39" s="6">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C39" s="6">
-        <v>2.42</v>
+        <v>2.38</v>
       </c>
       <c r="D39" s="6">
-        <v>141.49</v>
+        <v>140.65</v>
       </c>
       <c r="E39" s="6">
-        <v>202.12</v>
+        <v>200.94</v>
       </c>
       <c r="F39" s="6">
-        <v>909.55</v>
+        <v>904.21</v>
       </c>
       <c r="G39" s="6">
-        <v>303.18</v>
+        <v>301.4</v>
       </c>
       <c r="H39" s="6">
         <v>0</v>
@@ -4222,22 +4186,22 @@
         <v>81</v>
       </c>
       <c r="B40" s="6">
-        <v>147</v>
+        <v>130</v>
       </c>
       <c r="C40" s="6">
-        <v>2.45</v>
+        <v>2.17</v>
       </c>
       <c r="D40" s="6">
-        <v>135.12</v>
+        <v>137.42</v>
       </c>
       <c r="E40" s="6">
-        <v>193.03</v>
+        <v>196.31</v>
       </c>
       <c r="F40" s="6">
-        <v>868.66</v>
+        <v>883.41</v>
       </c>
       <c r="G40" s="6">
-        <v>289.55</v>
+        <v>294.47</v>
       </c>
       <c r="H40" s="6">
         <v>0</v>
@@ -4254,22 +4218,22 @@
         <v>82</v>
       </c>
       <c r="B41" s="6">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="C41" s="6">
-        <v>2.37</v>
+        <v>2.48</v>
       </c>
       <c r="D41" s="6">
-        <v>144</v>
+        <v>137.81</v>
       </c>
       <c r="E41" s="6">
-        <v>205.72</v>
+        <v>196.87</v>
       </c>
       <c r="F41" s="6">
-        <v>925.73</v>
+        <v>885.92</v>
       </c>
       <c r="G41" s="6">
-        <v>308.58</v>
+        <v>295.31</v>
       </c>
       <c r="H41" s="6">
         <v>0</v>
@@ -14773,7 +14737,7 @@
         <v>601</v>
       </c>
       <c r="E2" s="6">
-        <v>0</v>
+        <v>51.76</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -14790,7 +14754,7 @@
         <v>601</v>
       </c>
       <c r="E3" s="6">
-        <v>0</v>
+        <v>57.06</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -14807,7 +14771,7 @@
         <v>601</v>
       </c>
       <c r="E4" s="6">
-        <v>0</v>
+        <v>49.06</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -14824,7 +14788,7 @@
         <v>601</v>
       </c>
       <c r="E5" s="6">
-        <v>0</v>
+        <v>64.8</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -14841,7 +14805,7 @@
         <v>601</v>
       </c>
       <c r="E6" s="6">
-        <v>0</v>
+        <v>60.85</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -14858,7 +14822,7 @@
         <v>601</v>
       </c>
       <c r="E7" s="6">
-        <v>0</v>
+        <v>63.75</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -14875,7 +14839,7 @@
         <v>601</v>
       </c>
       <c r="E8" s="6">
-        <v>0</v>
+        <v>70.93</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -14892,7 +14856,7 @@
         <v>601</v>
       </c>
       <c r="E9" s="6">
-        <v>0</v>
+        <v>70.23</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -14909,7 +14873,7 @@
         <v>601</v>
       </c>
       <c r="E10" s="6">
-        <v>0</v>
+        <v>86.97</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -14926,7 +14890,7 @@
         <v>601</v>
       </c>
       <c r="E11" s="6">
-        <v>0</v>
+        <v>88.2</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -14943,7 +14907,7 @@
         <v>601</v>
       </c>
       <c r="E12" s="6">
-        <v>0</v>
+        <v>85.67</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -14960,7 +14924,7 @@
         <v>601</v>
       </c>
       <c r="E13" s="6">
-        <v>0</v>
+        <v>92.93</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -14977,7 +14941,7 @@
         <v>601</v>
       </c>
       <c r="E14" s="6">
-        <v>0</v>
+        <v>90.62</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -14994,7 +14958,7 @@
         <v>601</v>
       </c>
       <c r="E15" s="6">
-        <v>0</v>
+        <v>101.05</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -15011,7 +14975,7 @@
         <v>601</v>
       </c>
       <c r="E16" s="6">
-        <v>0</v>
+        <v>110.15</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -15028,7 +14992,7 @@
         <v>601</v>
       </c>
       <c r="E17" s="6">
-        <v>0</v>
+        <v>101.07</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -15045,7 +15009,7 @@
         <v>601</v>
       </c>
       <c r="E18" s="6">
-        <v>0</v>
+        <v>110.99</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -15062,7 +15026,7 @@
         <v>601</v>
       </c>
       <c r="E19" s="6">
-        <v>0</v>
+        <v>110.71</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -15079,7 +15043,7 @@
         <v>601</v>
       </c>
       <c r="E20" s="6">
-        <v>0</v>
+        <v>123.29</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -15096,7 +15060,7 @@
         <v>601</v>
       </c>
       <c r="E21" s="6">
-        <v>0</v>
+        <v>127.34</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -15113,7 +15077,7 @@
         <v>601</v>
       </c>
       <c r="E22" s="6">
-        <v>0</v>
+        <v>125.44</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -15130,7 +15094,7 @@
         <v>601</v>
       </c>
       <c r="E23" s="6">
-        <v>0</v>
+        <v>136.5</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -15147,7 +15111,7 @@
         <v>601</v>
       </c>
       <c r="E24" s="6">
-        <v>0</v>
+        <v>139.79</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -15164,7 +15128,7 @@
         <v>601</v>
       </c>
       <c r="E25" s="6">
-        <v>0</v>
+        <v>140.17</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -15181,7 +15145,7 @@
         <v>601</v>
       </c>
       <c r="E26" s="6">
-        <v>0</v>
+        <v>143.17</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -15198,7 +15162,7 @@
         <v>601</v>
       </c>
       <c r="E27" s="6">
-        <v>0</v>
+        <v>152.36</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -15215,7 +15179,7 @@
         <v>601</v>
       </c>
       <c r="E28" s="6">
-        <v>0</v>
+        <v>156.95</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -15232,7 +15196,7 @@
         <v>601</v>
       </c>
       <c r="E29" s="6">
-        <v>0</v>
+        <v>155.2</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -15249,7 +15213,7 @@
         <v>601</v>
       </c>
       <c r="E30" s="6">
-        <v>0</v>
+        <v>162.35</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -15266,29 +15230,29 @@
         <v>659</v>
       </c>
       <c r="E31" s="6">
-        <v>43.77</v>
+        <v>51.76</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="B32" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="D32" s="6" t="s">
         <v>601</v>
       </c>
       <c r="E32" s="6">
-        <v>0</v>
+        <v>165.82</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="B33" s="6" t="s">
         <v>599</v>
@@ -15297,32 +15261,32 @@
         <v>603</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="E33" s="6">
-        <v>52.68</v>
+        <v>57.06</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
-        <v>664</v>
+        <v>661</v>
       </c>
       <c r="B34" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>601</v>
       </c>
       <c r="E34" s="6">
-        <v>0</v>
+        <v>171.63</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="B35" s="6" t="s">
         <v>599</v>
@@ -15331,32 +15295,32 @@
         <v>605</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="E35" s="6">
-        <v>62.79</v>
+        <v>49.06</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
-        <v>668</v>
+        <v>664</v>
       </c>
       <c r="B36" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>601</v>
       </c>
       <c r="E36" s="6">
-        <v>0</v>
+        <v>164.94</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>599</v>
@@ -15365,32 +15329,32 @@
         <v>607</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>671</v>
+        <v>668</v>
       </c>
       <c r="E37" s="6">
-        <v>61.08</v>
+        <v>64.8</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
-        <v>672</v>
+        <v>667</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>673</v>
+        <v>669</v>
       </c>
       <c r="D38" s="6" t="s">
         <v>601</v>
       </c>
       <c r="E38" s="6">
-        <v>0</v>
+        <v>169.52</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
-        <v>674</v>
+        <v>670</v>
       </c>
       <c r="B39" s="6" t="s">
         <v>599</v>
@@ -15399,32 +15363,32 @@
         <v>609</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>675</v>
+        <v>671</v>
       </c>
       <c r="E39" s="6">
-        <v>68.02</v>
+        <v>60.85</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
-        <v>676</v>
+        <v>670</v>
       </c>
       <c r="B40" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>677</v>
+        <v>672</v>
       </c>
       <c r="D40" s="6" t="s">
         <v>601</v>
       </c>
       <c r="E40" s="6">
-        <v>0</v>
+        <v>174.35</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
-        <v>678</v>
+        <v>673</v>
       </c>
       <c r="B41" s="6" t="s">
         <v>599</v>
@@ -15433,32 +15397,32 @@
         <v>611</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>679</v>
+        <v>674</v>
       </c>
       <c r="E41" s="6">
-        <v>69.03</v>
+        <v>63.75</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
-        <v>680</v>
+        <v>673</v>
       </c>
       <c r="B42" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>681</v>
+        <v>675</v>
       </c>
       <c r="D42" s="6" t="s">
         <v>601</v>
       </c>
       <c r="E42" s="6">
-        <v>0</v>
+        <v>178.14</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
-        <v>682</v>
+        <v>676</v>
       </c>
       <c r="B43" s="6" t="s">
         <v>599</v>
@@ -15467,32 +15431,32 @@
         <v>613</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>683</v>
+        <v>677</v>
       </c>
       <c r="E43" s="6">
-        <v>78.53</v>
+        <v>70.93</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
-        <v>684</v>
+        <v>676</v>
       </c>
       <c r="B44" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>685</v>
+        <v>678</v>
       </c>
       <c r="D44" s="6" t="s">
         <v>601</v>
       </c>
       <c r="E44" s="6">
-        <v>0</v>
+        <v>180.15</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
-        <v>686</v>
+        <v>679</v>
       </c>
       <c r="B45" s="6" t="s">
         <v>599</v>
@@ -15501,32 +15465,32 @@
         <v>615</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>687</v>
+        <v>680</v>
       </c>
       <c r="E45" s="6">
-        <v>79.89</v>
+        <v>70.23</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
-        <v>688</v>
+        <v>679</v>
       </c>
       <c r="B46" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>689</v>
+        <v>681</v>
       </c>
       <c r="D46" s="6" t="s">
         <v>601</v>
       </c>
       <c r="E46" s="6">
-        <v>0</v>
+        <v>195.82</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
-        <v>690</v>
+        <v>682</v>
       </c>
       <c r="B47" s="6" t="s">
         <v>599</v>
@@ -15535,32 +15499,32 @@
         <v>617</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>691</v>
+        <v>683</v>
       </c>
       <c r="E47" s="6">
-        <v>81.09</v>
+        <v>86.97</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
-        <v>692</v>
+        <v>682</v>
       </c>
       <c r="B48" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>693</v>
+        <v>684</v>
       </c>
       <c r="D48" s="6" t="s">
         <v>601</v>
       </c>
       <c r="E48" s="6">
-        <v>0</v>
+        <v>192.78</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
-        <v>694</v>
+        <v>685</v>
       </c>
       <c r="B49" s="6" t="s">
         <v>599</v>
@@ -15569,32 +15533,32 @@
         <v>619</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>695</v>
+        <v>686</v>
       </c>
       <c r="E49" s="6">
-        <v>87.28</v>
+        <v>88.2</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
-        <v>696</v>
+        <v>685</v>
       </c>
       <c r="B50" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>697</v>
+        <v>687</v>
       </c>
       <c r="D50" s="6" t="s">
         <v>601</v>
       </c>
       <c r="E50" s="6">
-        <v>0</v>
+        <v>206.94</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
-        <v>698</v>
+        <v>688</v>
       </c>
       <c r="B51" s="6" t="s">
         <v>599</v>
@@ -15603,32 +15567,32 @@
         <v>621</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>699</v>
+        <v>689</v>
       </c>
       <c r="E51" s="6">
-        <v>90.48</v>
+        <v>85.67</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
-        <v>700</v>
+        <v>688</v>
       </c>
       <c r="B52" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>701</v>
+        <v>690</v>
       </c>
       <c r="D52" s="6" t="s">
         <v>601</v>
       </c>
       <c r="E52" s="6">
-        <v>0</v>
+        <v>209.05</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
-        <v>702</v>
+        <v>691</v>
       </c>
       <c r="B53" s="6" t="s">
         <v>599</v>
@@ -15637,15 +15601,15 @@
         <v>623</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>703</v>
+        <v>692</v>
       </c>
       <c r="E53" s="6">
-        <v>98.14</v>
+        <v>92.93</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
-        <v>704</v>
+        <v>693</v>
       </c>
       <c r="B54" s="6" t="s">
         <v>599</v>
@@ -15654,15 +15618,15 @@
         <v>625</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>705</v>
+        <v>694</v>
       </c>
       <c r="E54" s="6">
-        <v>94.56</v>
+        <v>90.62</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
-        <v>706</v>
+        <v>695</v>
       </c>
       <c r="B55" s="6" t="s">
         <v>599</v>
@@ -15671,15 +15635,15 @@
         <v>627</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>707</v>
+        <v>696</v>
       </c>
       <c r="E55" s="6">
-        <v>101.17</v>
+        <v>101.05</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
-        <v>708</v>
+        <v>697</v>
       </c>
       <c r="B56" s="6" t="s">
         <v>599</v>
@@ -15688,15 +15652,15 @@
         <v>629</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>709</v>
+        <v>698</v>
       </c>
       <c r="E56" s="6">
-        <v>106.52</v>
+        <v>110.15</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
-        <v>710</v>
+        <v>699</v>
       </c>
       <c r="B57" s="6" t="s">
         <v>599</v>
@@ -15705,15 +15669,15 @@
         <v>631</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>711</v>
+        <v>700</v>
       </c>
       <c r="E57" s="6">
-        <v>100.06</v>
+        <v>101.07</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
-        <v>712</v>
+        <v>701</v>
       </c>
       <c r="B58" s="6" t="s">
         <v>599</v>
@@ -15722,15 +15686,15 @@
         <v>633</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>713</v>
+        <v>702</v>
       </c>
       <c r="E58" s="6">
-        <v>104.45</v>
+        <v>110.99</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
-        <v>714</v>
+        <v>703</v>
       </c>
       <c r="B59" s="6" t="s">
         <v>599</v>
@@ -15739,15 +15703,15 @@
         <v>635</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>715</v>
+        <v>704</v>
       </c>
       <c r="E59" s="6">
-        <v>108.45</v>
+        <v>110.71</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
-        <v>716</v>
+        <v>705</v>
       </c>
       <c r="B60" s="6" t="s">
         <v>599</v>
@@ -15756,15 +15720,15 @@
         <v>637</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>717</v>
+        <v>706</v>
       </c>
       <c r="E60" s="6">
-        <v>125.97</v>
+        <v>123.29</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
-        <v>718</v>
+        <v>707</v>
       </c>
       <c r="B61" s="6" t="s">
         <v>599</v>
@@ -15773,15 +15737,15 @@
         <v>639</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>719</v>
+        <v>708</v>
       </c>
       <c r="E61" s="6">
-        <v>124.22</v>
+        <v>127.34</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
-        <v>720</v>
+        <v>709</v>
       </c>
       <c r="B62" s="6" t="s">
         <v>599</v>
@@ -15790,15 +15754,15 @@
         <v>641</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>721</v>
+        <v>710</v>
       </c>
       <c r="E62" s="6">
-        <v>120.25</v>
+        <v>125.44</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
-        <v>722</v>
+        <v>711</v>
       </c>
       <c r="B63" s="6" t="s">
         <v>599</v>
@@ -15807,15 +15771,15 @@
         <v>643</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>723</v>
+        <v>712</v>
       </c>
       <c r="E63" s="6">
-        <v>126.5</v>
+        <v>136.5</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
-        <v>724</v>
+        <v>713</v>
       </c>
       <c r="B64" s="6" t="s">
         <v>599</v>
@@ -15824,15 +15788,15 @@
         <v>645</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>725</v>
+        <v>714</v>
       </c>
       <c r="E64" s="6">
-        <v>133.25</v>
+        <v>139.79</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
-        <v>726</v>
+        <v>715</v>
       </c>
       <c r="B65" s="6" t="s">
         <v>599</v>
@@ -15841,15 +15805,15 @@
         <v>647</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>727</v>
+        <v>716</v>
       </c>
       <c r="E65" s="6">
-        <v>141.98</v>
+        <v>140.17</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
-        <v>728</v>
+        <v>717</v>
       </c>
       <c r="B66" s="6" t="s">
         <v>599</v>
@@ -15858,15 +15822,15 @@
         <v>649</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>729</v>
+        <v>718</v>
       </c>
       <c r="E66" s="6">
-        <v>140.79</v>
+        <v>143.17</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
-        <v>730</v>
+        <v>719</v>
       </c>
       <c r="B67" s="6" t="s">
         <v>599</v>
@@ -15875,15 +15839,15 @@
         <v>651</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>731</v>
+        <v>720</v>
       </c>
       <c r="E67" s="6">
-        <v>150.42</v>
+        <v>152.36</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
-        <v>732</v>
+        <v>721</v>
       </c>
       <c r="B68" s="6" t="s">
         <v>599</v>
@@ -15892,15 +15856,15 @@
         <v>653</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>733</v>
+        <v>722</v>
       </c>
       <c r="E68" s="6">
-        <v>150.77</v>
+        <v>156.95</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
-        <v>734</v>
+        <v>723</v>
       </c>
       <c r="B69" s="6" t="s">
         <v>599</v>
@@ -15909,15 +15873,15 @@
         <v>655</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>735</v>
+        <v>724</v>
       </c>
       <c r="E69" s="6">
-        <v>153.02</v>
+        <v>155.2</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
-        <v>736</v>
+        <v>725</v>
       </c>
       <c r="B70" s="6" t="s">
         <v>599</v>
@@ -15926,15 +15890,15 @@
         <v>657</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>737</v>
+        <v>726</v>
       </c>
       <c r="E70" s="6">
-        <v>164.45</v>
+        <v>162.35</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
-        <v>738</v>
+        <v>727</v>
       </c>
       <c r="B71" s="6" t="s">
         <v>599</v>
@@ -15943,15 +15907,15 @@
         <v>600</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E71" s="6">
-        <v>43.77</v>
+        <v>51.76</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
-        <v>738</v>
+        <v>727</v>
       </c>
       <c r="B72" s="6" t="s">
         <v>599</v>
@@ -15960,15 +15924,15 @@
         <v>603</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E72" s="6">
-        <v>52.68</v>
+        <v>57.06</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
-        <v>738</v>
+        <v>727</v>
       </c>
       <c r="B73" s="6" t="s">
         <v>599</v>
@@ -15977,15 +15941,15 @@
         <v>605</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E73" s="6">
-        <v>62.79</v>
+        <v>49.06</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
-        <v>738</v>
+        <v>727</v>
       </c>
       <c r="B74" s="6" t="s">
         <v>599</v>
@@ -15994,15 +15958,15 @@
         <v>607</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E74" s="6">
-        <v>61.08</v>
+        <v>64.8</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
-        <v>738</v>
+        <v>727</v>
       </c>
       <c r="B75" s="6" t="s">
         <v>599</v>
@@ -16011,15 +15975,15 @@
         <v>609</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E75" s="6">
-        <v>68.02</v>
+        <v>60.85</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
-        <v>738</v>
+        <v>727</v>
       </c>
       <c r="B76" s="6" t="s">
         <v>599</v>
@@ -16028,15 +15992,15 @@
         <v>611</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E76" s="6">
-        <v>69.03</v>
+        <v>63.75</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
-        <v>738</v>
+        <v>727</v>
       </c>
       <c r="B77" s="6" t="s">
         <v>599</v>
@@ -16045,15 +16009,15 @@
         <v>613</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E77" s="6">
-        <v>78.53</v>
+        <v>70.93</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
-        <v>738</v>
+        <v>727</v>
       </c>
       <c r="B78" s="6" t="s">
         <v>599</v>
@@ -16062,15 +16026,15 @@
         <v>615</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E78" s="6">
-        <v>79.89</v>
+        <v>70.23</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="6" t="s">
-        <v>738</v>
+        <v>727</v>
       </c>
       <c r="B79" s="6" t="s">
         <v>599</v>
@@ -16079,15 +16043,15 @@
         <v>617</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E79" s="6">
-        <v>81.09</v>
+        <v>86.97</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="6" t="s">
-        <v>738</v>
+        <v>727</v>
       </c>
       <c r="B80" s="6" t="s">
         <v>599</v>
@@ -16096,15 +16060,15 @@
         <v>619</v>
       </c>
       <c r="D80" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E80" s="6">
-        <v>87.28</v>
+        <v>88.2</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B81" s="6" t="s">
         <v>599</v>
@@ -16113,15 +16077,15 @@
         <v>621</v>
       </c>
       <c r="D81" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E81" s="6">
-        <v>90.48</v>
+        <v>85.67</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B82" s="6" t="s">
         <v>599</v>
@@ -16130,15 +16094,15 @@
         <v>623</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E82" s="6">
-        <v>98.14</v>
+        <v>92.93</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B83" s="6" t="s">
         <v>599</v>
@@ -16147,15 +16111,15 @@
         <v>625</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E83" s="6">
-        <v>94.56</v>
+        <v>90.62</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B84" s="6" t="s">
         <v>599</v>
@@ -16164,15 +16128,15 @@
         <v>627</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E84" s="6">
-        <v>101.17</v>
+        <v>101.05</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B85" s="6" t="s">
         <v>599</v>
@@ -16181,15 +16145,15 @@
         <v>629</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E85" s="6">
-        <v>106.52</v>
+        <v>110.15</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B86" s="6" t="s">
         <v>599</v>
@@ -16198,15 +16162,15 @@
         <v>631</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E86" s="6">
-        <v>100.06</v>
+        <v>101.07</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B87" s="6" t="s">
         <v>599</v>
@@ -16215,15 +16179,15 @@
         <v>633</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E87" s="6">
-        <v>104.45</v>
+        <v>110.99</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B88" s="6" t="s">
         <v>599</v>
@@ -16232,15 +16196,15 @@
         <v>635</v>
       </c>
       <c r="D88" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E88" s="6">
-        <v>108.45</v>
+        <v>110.71</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B89" s="6" t="s">
         <v>599</v>
@@ -16249,15 +16213,15 @@
         <v>637</v>
       </c>
       <c r="D89" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E89" s="6">
-        <v>125.97</v>
+        <v>123.29</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B90" s="6" t="s">
         <v>599</v>
@@ -16266,15 +16230,15 @@
         <v>639</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E90" s="6">
-        <v>124.22</v>
+        <v>127.34</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B91" s="6" t="s">
         <v>599</v>
@@ -16283,15 +16247,15 @@
         <v>641</v>
       </c>
       <c r="D91" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E91" s="6">
-        <v>120.25</v>
+        <v>125.44</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B92" s="6" t="s">
         <v>599</v>
@@ -16300,15 +16264,15 @@
         <v>643</v>
       </c>
       <c r="D92" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E92" s="6">
-        <v>126.5</v>
+        <v>136.5</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B93" s="6" t="s">
         <v>599</v>
@@ -16317,15 +16281,15 @@
         <v>645</v>
       </c>
       <c r="D93" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E93" s="6">
-        <v>133.25</v>
+        <v>139.79</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B94" s="6" t="s">
         <v>599</v>
@@ -16334,15 +16298,15 @@
         <v>647</v>
       </c>
       <c r="D94" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E94" s="6">
-        <v>141.98</v>
+        <v>140.17</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B95" s="6" t="s">
         <v>599</v>
@@ -16351,15 +16315,15 @@
         <v>649</v>
       </c>
       <c r="D95" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E95" s="6">
-        <v>140.79</v>
+        <v>143.17</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B96" s="6" t="s">
         <v>599</v>
@@ -16368,15 +16332,15 @@
         <v>651</v>
       </c>
       <c r="D96" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E96" s="6">
-        <v>150.42</v>
+        <v>152.36</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B97" s="6" t="s">
         <v>599</v>
@@ -16385,15 +16349,15 @@
         <v>653</v>
       </c>
       <c r="D97" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E97" s="6">
-        <v>150.77</v>
+        <v>156.95</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B98" s="6" t="s">
         <v>599</v>
@@ -16402,15 +16366,15 @@
         <v>655</v>
       </c>
       <c r="D98" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E98" s="6">
-        <v>153.02</v>
+        <v>155.2</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B99" s="6" t="s">
         <v>599</v>
@@ -16419,384 +16383,384 @@
         <v>657</v>
       </c>
       <c r="D99" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E99" s="6">
-        <v>164.45</v>
+        <v>162.35</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B100" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C100" s="6" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="D100" s="6" t="s">
-        <v>741</v>
+        <v>729</v>
       </c>
       <c r="E100" s="6">
-        <v>164.88</v>
+        <v>165.82</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B101" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C101" s="6" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="D101" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E101" s="6">
-        <v>164.88</v>
+        <v>165.82</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B102" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C102" s="6" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="D102" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E102" s="6">
-        <v>169.04</v>
+        <v>171.63</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B103" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C103" s="6" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="D103" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E103" s="6">
-        <v>173.34</v>
+        <v>164.94</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B104" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C104" s="6" t="s">
-        <v>673</v>
+        <v>669</v>
       </c>
       <c r="D104" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E104" s="6">
-        <v>168.54</v>
+        <v>169.52</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B105" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C105" s="6" t="s">
-        <v>677</v>
+        <v>672</v>
       </c>
       <c r="D105" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E105" s="6">
-        <v>184.69</v>
+        <v>174.35</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B106" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C106" s="6" t="s">
-        <v>681</v>
+        <v>675</v>
       </c>
       <c r="D106" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E106" s="6">
-        <v>185.31</v>
+        <v>178.14</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B107" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C107" s="6" t="s">
-        <v>685</v>
+        <v>678</v>
       </c>
       <c r="D107" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E107" s="6">
-        <v>190.74</v>
+        <v>180.15</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B108" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C108" s="6" t="s">
-        <v>689</v>
+        <v>681</v>
       </c>
       <c r="D108" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E108" s="6">
-        <v>184.36</v>
+        <v>195.82</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B109" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C109" s="6" t="s">
-        <v>693</v>
+        <v>684</v>
       </c>
       <c r="D109" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E109" s="6">
-        <v>200.26</v>
+        <v>192.78</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B110" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C110" s="6" t="s">
-        <v>697</v>
+        <v>687</v>
       </c>
       <c r="D110" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E110" s="6">
-        <v>196.44</v>
+        <v>206.94</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="6" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="B111" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C111" s="6" t="s">
-        <v>701</v>
+        <v>690</v>
       </c>
       <c r="D111" s="6" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="E111" s="6">
-        <v>201.94</v>
+        <v>209.05</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" s="6" t="s">
-        <v>742</v>
+        <v>730</v>
       </c>
       <c r="B112" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C112" s="6" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="D112" s="6" t="s">
-        <v>743</v>
+        <v>731</v>
       </c>
       <c r="E112" s="6">
-        <v>169.04</v>
+        <v>171.63</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="6" t="s">
-        <v>744</v>
+        <v>732</v>
       </c>
       <c r="B113" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C113" s="6" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="D113" s="6" t="s">
-        <v>745</v>
+        <v>733</v>
       </c>
       <c r="E113" s="6">
-        <v>173.34</v>
+        <v>164.94</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="6" t="s">
-        <v>746</v>
+        <v>734</v>
       </c>
       <c r="B114" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C114" s="6" t="s">
-        <v>673</v>
+        <v>669</v>
       </c>
       <c r="D114" s="6" t="s">
-        <v>747</v>
+        <v>735</v>
       </c>
       <c r="E114" s="6">
-        <v>168.54</v>
+        <v>169.52</v>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="6" t="s">
-        <v>748</v>
+        <v>736</v>
       </c>
       <c r="B115" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C115" s="6" t="s">
-        <v>677</v>
+        <v>672</v>
       </c>
       <c r="D115" s="6" t="s">
-        <v>749</v>
+        <v>737</v>
       </c>
       <c r="E115" s="6">
-        <v>184.69</v>
+        <v>174.35</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="6" t="s">
-        <v>750</v>
+        <v>738</v>
       </c>
       <c r="B116" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C116" s="6" t="s">
-        <v>681</v>
+        <v>675</v>
       </c>
       <c r="D116" s="6" t="s">
-        <v>751</v>
+        <v>739</v>
       </c>
       <c r="E116" s="6">
-        <v>185.31</v>
+        <v>178.14</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="6" t="s">
-        <v>752</v>
+        <v>740</v>
       </c>
       <c r="B117" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C117" s="6" t="s">
-        <v>685</v>
+        <v>678</v>
       </c>
       <c r="D117" s="6" t="s">
-        <v>753</v>
+        <v>741</v>
       </c>
       <c r="E117" s="6">
-        <v>190.74</v>
+        <v>180.15</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="6" t="s">
-        <v>754</v>
+        <v>742</v>
       </c>
       <c r="B118" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C118" s="6" t="s">
-        <v>689</v>
+        <v>681</v>
       </c>
       <c r="D118" s="6" t="s">
-        <v>755</v>
+        <v>743</v>
       </c>
       <c r="E118" s="6">
-        <v>184.36</v>
+        <v>195.82</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="6" t="s">
-        <v>756</v>
+        <v>744</v>
       </c>
       <c r="B119" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C119" s="6" t="s">
-        <v>693</v>
+        <v>684</v>
       </c>
       <c r="D119" s="6" t="s">
-        <v>757</v>
+        <v>745</v>
       </c>
       <c r="E119" s="6">
-        <v>200.26</v>
+        <v>192.78</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="6" t="s">
-        <v>758</v>
+        <v>746</v>
       </c>
       <c r="B120" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C120" s="6" t="s">
-        <v>697</v>
+        <v>687</v>
       </c>
       <c r="D120" s="6" t="s">
-        <v>759</v>
+        <v>747</v>
       </c>
       <c r="E120" s="6">
-        <v>196.44</v>
+        <v>206.94</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="6" t="s">
-        <v>760</v>
+        <v>748</v>
       </c>
       <c r="B121" s="6" t="s">
         <v>599</v>
       </c>
       <c r="C121" s="6" t="s">
-        <v>701</v>
+        <v>690</v>
       </c>
       <c r="D121" s="6" t="s">
-        <v>761</v>
+        <v>749</v>
       </c>
       <c r="E121" s="6">
-        <v>201.94</v>
+        <v>209.05</v>
       </c>
     </row>
   </sheetData>

</xml_diff>